<commit_message>
Update Range Collection H1 tags (about 90 IDs looked up)
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Number is an Encompass item ID, not a manufacturer part number; no web page found for it</t>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -931,222 +931,254 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="2" t="n">
         <v>9441452</v>
       </c>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>W10314417</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Panel Assembly - W10314417</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9441452; single Encompass page</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="3" t="n">
         <v>11436677</v>
       </c>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B22" s="4" t="n">
+      <c r="B22" s="3" t="n">
         <v>10157279</v>
       </c>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="3" t="n">
         <v>10611794</v>
       </c>
-      <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B24" s="4" t="n">
+      <c r="B24" s="3" t="n">
         <v>10886963</v>
       </c>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n">
+      <c r="B25" s="2" t="n">
         <v>11435391</v>
       </c>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>W11050551</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Board - W11050551</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 11435391; single Encompass page</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n">
+      <c r="B26" s="2" t="n">
         <v>9441394</v>
       </c>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>WPW10312660</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Gas Control Board - WPW10312660</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9441394; single Encompass page</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n">
+      <c r="B27" s="3" t="n">
         <v>11436042</v>
       </c>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n">
+      <c r="B28" s="3" t="n">
         <v>11435736</v>
       </c>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="2" t="n">
         <v>11435125</v>
       </c>
-      <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>W11039099</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Electronic Oven Control Board - W11039099</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 11435125; single Encompass page</t>
         </is>
       </c>
     </row>
@@ -1173,24 +1205,32 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n">
+      <c r="B31" s="3" t="n">
         <v>10891704</v>
       </c>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>W10814036</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Whirlpool Cooktop Cooktop Main Top - W10814036</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 10891704; listing name only "Cooktop"</t>
         </is>
       </c>
     </row>
@@ -1283,68 +1323,84 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B36" s="4" t="n">
+      <c r="B36" s="2" t="n">
         <v>10886716</v>
       </c>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>W10884488</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Board - W10884488</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 10886716; two Encompass pages</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B37" s="4" t="n">
+      <c r="B37" s="3" t="n">
         <v>10886968</v>
       </c>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B38" s="4" t="n">
+      <c r="B38" s="2" t="n">
         <v>10886969</v>
       </c>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr"/>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>W10904904</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Electronic Control Board - W10904904</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 10886969; single Encompass page</t>
         </is>
       </c>
     </row>
@@ -1459,112 +1515,128 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B44" s="4" t="n">
+      <c r="B44" s="3" t="n">
         <v>10610180</v>
       </c>
-      <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B45" s="4" t="n">
+      <c r="B45" s="2" t="n">
         <v>10610337</v>
       </c>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>WPW10778305</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Oven Control Board - WPW10778305</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 10610337 (SP10610337 cross-reference)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B46" s="4" t="n">
+      <c r="B46" s="3" t="n">
         <v>10600408</v>
       </c>
-      <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B47" s="4" t="n">
+      <c r="B47" s="2" t="n">
         <v>10611938</v>
       </c>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>W10772617</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Washer Outer Tub - W10772617</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 10611938; two Encompass pages</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B48" s="4" t="n">
+      <c r="B48" s="3" t="n">
         <v>10611357</v>
       </c>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -1701,24 +1773,24 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B55" s="4" t="n">
+      <c r="B55" s="3" t="n">
         <v>9435695</v>
       </c>
-      <c r="C55" s="4" t="inlineStr"/>
-      <c r="D55" s="4" t="inlineStr"/>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -2691,46 +2763,62 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="inlineStr">
+      <c r="A100" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B100" s="4" t="n">
+      <c r="B100" s="3" t="n">
         <v>11574168</v>
       </c>
-      <c r="C100" s="4" t="inlineStr"/>
-      <c r="D100" s="4" t="inlineStr"/>
-      <c r="E100" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F100" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>W11178790</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>Whirlpool Cooktop Cooktop Main Top - W11178790</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 11574168; listing name only "Cooktop"</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="4" t="inlineStr">
+      <c r="A101" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B101" s="4" t="n">
+      <c r="B101" s="2" t="n">
         <v>12276720</v>
       </c>
-      <c r="C101" s="4" t="inlineStr"/>
-      <c r="D101" s="4" t="inlineStr"/>
-      <c r="E101" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F101" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>W11219379</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Oven Glass Door - W11219379</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 12276720; two pages</t>
         </is>
       </c>
     </row>
@@ -2955,90 +3043,90 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="4" t="inlineStr">
+      <c r="A112" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B112" s="4" t="n">
+      <c r="B112" s="3" t="n">
         <v>12329123</v>
       </c>
-      <c r="C112" s="4" t="inlineStr"/>
-      <c r="D112" s="4" t="inlineStr"/>
-      <c r="E112" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F112" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C112" s="3" t="inlineStr"/>
+      <c r="D112" s="3" t="inlineStr"/>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="4" t="inlineStr">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B113" s="4" t="n">
+      <c r="B113" s="3" t="n">
         <v>11433914</v>
       </c>
-      <c r="C113" s="4" t="inlineStr"/>
-      <c r="D113" s="4" t="inlineStr"/>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C113" s="3" t="inlineStr"/>
+      <c r="D113" s="3" t="inlineStr"/>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="4" t="inlineStr">
+      <c r="A114" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B114" s="4" t="n">
+      <c r="B114" s="3" t="n">
         <v>11435787</v>
       </c>
-      <c r="C114" s="4" t="inlineStr"/>
-      <c r="D114" s="4" t="inlineStr"/>
-      <c r="E114" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F114" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C114" s="3" t="inlineStr"/>
+      <c r="D114" s="3" t="inlineStr"/>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="4" t="inlineStr">
+      <c r="A115" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B115" s="4" t="n">
+      <c r="B115" s="3" t="n">
         <v>10611282</v>
       </c>
-      <c r="C115" s="4" t="inlineStr"/>
-      <c r="D115" s="4" t="inlineStr"/>
-      <c r="E115" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F115" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C115" s="3" t="inlineStr"/>
+      <c r="D115" s="3" t="inlineStr"/>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -3065,90 +3153,98 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="4" t="inlineStr">
+      <c r="A117" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B117" s="4" t="n">
+      <c r="B117" s="2" t="n">
         <v>11434431</v>
       </c>
-      <c r="C117" s="4" t="inlineStr"/>
-      <c r="D117" s="4" t="inlineStr"/>
-      <c r="E117" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F117" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>W10919303</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Panel - W10919303</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 11434431; single page</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="4" t="inlineStr">
+      <c r="A118" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B118" s="4" t="n">
+      <c r="B118" s="3" t="n">
         <v>11432514</v>
       </c>
-      <c r="C118" s="4" t="inlineStr"/>
-      <c r="D118" s="4" t="inlineStr"/>
-      <c r="E118" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F118" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C118" s="3" t="inlineStr"/>
+      <c r="D118" s="3" t="inlineStr"/>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="4" t="inlineStr">
+      <c r="A119" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B119" s="4" t="n">
+      <c r="B119" s="3" t="n">
         <v>11432299</v>
       </c>
-      <c r="C119" s="4" t="inlineStr"/>
-      <c r="D119" s="4" t="inlineStr"/>
-      <c r="E119" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F119" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C119" s="3" t="inlineStr"/>
+      <c r="D119" s="3" t="inlineStr"/>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="4" t="inlineStr">
+      <c r="A120" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B120" s="4" t="n">
+      <c r="B120" s="3" t="n">
         <v>9442266</v>
       </c>
-      <c r="C120" s="4" t="inlineStr"/>
-      <c r="D120" s="4" t="inlineStr"/>
-      <c r="E120" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F120" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C120" s="3" t="inlineStr"/>
+      <c r="D120" s="3" t="inlineStr"/>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -4077,112 +4173,120 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="4" t="inlineStr">
+      <c r="A163" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B163" s="4" t="n">
+      <c r="B163" s="3" t="n">
         <v>9892353</v>
       </c>
-      <c r="C163" s="4" t="inlineStr"/>
-      <c r="D163" s="4" t="inlineStr"/>
-      <c r="E163" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F163" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C163" s="3" t="inlineStr"/>
+      <c r="D163" s="3" t="inlineStr"/>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="4" t="inlineStr">
+      <c r="A164" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B164" s="4" t="n">
+      <c r="B164" s="3" t="n">
         <v>9892346</v>
       </c>
-      <c r="C164" s="4" t="inlineStr"/>
-      <c r="D164" s="4" t="inlineStr"/>
-      <c r="E164" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F164" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C164" s="3" t="inlineStr"/>
+      <c r="D164" s="3" t="inlineStr"/>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="4" t="inlineStr">
+      <c r="A165" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B165" s="4" t="n">
+      <c r="B165" s="3" t="n">
         <v>9890274</v>
       </c>
-      <c r="C165" s="4" t="inlineStr"/>
-      <c r="D165" s="4" t="inlineStr"/>
-      <c r="E165" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F165" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C165" s="3" t="inlineStr"/>
+      <c r="D165" s="3" t="inlineStr"/>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="4" t="inlineStr">
+      <c r="A166" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B166" s="4" t="n">
+      <c r="B166" s="2" t="n">
         <v>9889686</v>
       </c>
-      <c r="C166" s="4" t="inlineStr"/>
-      <c r="D166" s="4" t="inlineStr"/>
-      <c r="E166" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F166" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>WPW10586736</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Oven Control Board - WPW10586736</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9889686; two pages</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="4" t="inlineStr">
+      <c r="A167" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B167" s="4" t="n">
+      <c r="B167" s="3" t="n">
         <v>9884707</v>
       </c>
-      <c r="C167" s="4" t="inlineStr"/>
-      <c r="D167" s="4" t="inlineStr"/>
-      <c r="E167" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F167" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C167" s="3" t="inlineStr"/>
+      <c r="D167" s="3" t="inlineStr"/>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -4231,288 +4335,344 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="4" t="inlineStr">
+      <c r="A170" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B170" s="4" t="n">
+      <c r="B170" s="3" t="n">
         <v>9443754</v>
       </c>
-      <c r="C170" s="4" t="inlineStr"/>
-      <c r="D170" s="4" t="inlineStr"/>
-      <c r="E170" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F170" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>WPW10396829</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>Whirlpool Cooktop Cooktop Main Top - WPW10396829</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9443754; listing name only "Cooktop"</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="4" t="inlineStr">
+      <c r="A171" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B171" s="4" t="n">
+      <c r="B171" s="2" t="n">
         <v>9443235</v>
       </c>
-      <c r="C171" s="4" t="inlineStr"/>
-      <c r="D171" s="4" t="inlineStr"/>
-      <c r="E171" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F171" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>W10365134</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Glass Main Top - W10365134</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9443235; single page</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="4" t="inlineStr">
+      <c r="A172" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B172" s="4" t="n">
+      <c r="B172" s="2" t="n">
         <v>9442761</v>
       </c>
-      <c r="C172" s="4" t="inlineStr"/>
-      <c r="D172" s="4" t="inlineStr"/>
-      <c r="E172" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F172" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>WPW10349742</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Electronic Control Board - WPW10349742</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9442761; single page (LCC195 board)</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="4" t="inlineStr">
+      <c r="A173" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B173" s="4" t="n">
+      <c r="B173" s="3" t="n">
         <v>9442710</v>
       </c>
-      <c r="C173" s="4" t="inlineStr"/>
-      <c r="D173" s="4" t="inlineStr"/>
-      <c r="E173" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F173" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C173" s="3" t="inlineStr"/>
+      <c r="D173" s="3" t="inlineStr"/>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="4" t="inlineStr">
+      <c r="A174" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B174" s="4" t="n">
+      <c r="B174" s="3" t="n">
         <v>9441456</v>
       </c>
-      <c r="C174" s="4" t="inlineStr"/>
-      <c r="D174" s="4" t="inlineStr"/>
-      <c r="E174" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F174" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C174" s="3" t="inlineStr"/>
+      <c r="D174" s="3" t="inlineStr"/>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="4" t="inlineStr">
+      <c r="A175" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B175" s="4" t="n">
+      <c r="B175" s="3" t="n">
         <v>9441453</v>
       </c>
-      <c r="C175" s="4" t="inlineStr"/>
-      <c r="D175" s="4" t="inlineStr"/>
-      <c r="E175" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F175" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C175" s="3" t="inlineStr"/>
+      <c r="D175" s="3" t="inlineStr"/>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="4" t="inlineStr">
+      <c r="A176" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B176" s="4" t="n">
+      <c r="B176" s="2" t="n">
         <v>9440666</v>
       </c>
-      <c r="C176" s="4" t="inlineStr"/>
-      <c r="D176" s="4" t="inlineStr"/>
-      <c r="E176" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F176" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>WPW10293048</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Gas Valve 4" - WPW10293048</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9440666; single page</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="4" t="inlineStr">
+      <c r="A177" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B177" s="4" t="n">
+      <c r="B177" s="3" t="n">
         <v>9439424</v>
       </c>
-      <c r="C177" s="4" t="inlineStr"/>
-      <c r="D177" s="4" t="inlineStr"/>
-      <c r="E177" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F177" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C177" s="3" t="inlineStr"/>
+      <c r="D177" s="3" t="inlineStr"/>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="4" t="inlineStr">
+      <c r="A178" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B178" s="4" t="n">
+      <c r="B178" s="3" t="n">
         <v>9439422</v>
       </c>
-      <c r="C178" s="4" t="inlineStr"/>
-      <c r="D178" s="4" t="inlineStr"/>
-      <c r="E178" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F178" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C178" s="3" t="inlineStr"/>
+      <c r="D178" s="3" t="inlineStr"/>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="4" t="inlineStr">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B179" s="4" t="n">
+      <c r="B179" s="2" t="n">
         <v>9415744</v>
       </c>
-      <c r="C179" s="4" t="inlineStr"/>
-      <c r="D179" s="4" t="inlineStr"/>
-      <c r="E179" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F179" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>WP8507P236-60</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Oven Control Board - WP8507P236-60</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9415744; single page</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="4" t="inlineStr">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B180" s="4" t="n">
+      <c r="B180" s="2" t="n">
         <v>9415741</v>
       </c>
-      <c r="C180" s="4" t="inlineStr"/>
-      <c r="D180" s="4" t="inlineStr"/>
-      <c r="E180" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F180" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>WP8507P231-60</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Board - WP8507P231-60</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9415741; two pages</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="4" t="inlineStr">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B181" s="4" t="n">
+      <c r="B181" s="2" t="n">
         <v>9415739</v>
       </c>
-      <c r="C181" s="4" t="inlineStr"/>
-      <c r="D181" s="4" t="inlineStr"/>
-      <c r="E181" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F181" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>WP8507P229-60</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Oven Control Board - WP8507P229-60</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9415739; single page</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="4" t="inlineStr">
+      <c r="A182" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B182" s="4" t="n">
+      <c r="B182" s="3" t="n">
         <v>9415736</v>
       </c>
-      <c r="C182" s="4" t="inlineStr"/>
-      <c r="D182" s="4" t="inlineStr"/>
-      <c r="E182" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F182" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C182" s="3" t="inlineStr"/>
+      <c r="D182" s="3" t="inlineStr"/>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -4539,46 +4699,62 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="4" t="inlineStr">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B184" s="4" t="n">
+      <c r="B184" s="2" t="n">
         <v>9394490</v>
       </c>
-      <c r="C184" s="4" t="inlineStr"/>
-      <c r="D184" s="4" t="inlineStr"/>
-      <c r="E184" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F184" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>WP5760M302-60</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Overlay Assembly - WP5760M302-60</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9394490; single page</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="4" t="inlineStr">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B185" s="4" t="n">
+      <c r="B185" s="2" t="n">
         <v>9250850</v>
       </c>
-      <c r="C185" s="4" t="inlineStr"/>
-      <c r="D185" s="4" t="inlineStr"/>
-      <c r="E185" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F185" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>5701M760-60</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Oven Control Board &amp; Clock Overlay Kit - 5701M760-60</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9250850; single page (Maytag-branded)</t>
         </is>
       </c>
     </row>
@@ -4671,46 +4847,62 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="4" t="inlineStr">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B190" s="4" t="n">
+      <c r="B190" s="2" t="n">
         <v>7038738</v>
       </c>
-      <c r="C190" s="4" t="inlineStr"/>
-      <c r="D190" s="4" t="inlineStr"/>
-      <c r="E190" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F190" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>WP9763716</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Gas Pressure Regulator &amp; Safety Valve - WP9763716</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 7038738; Encompass and Amazon pages</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="4" t="inlineStr">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B191" s="4" t="n">
+      <c r="B191" s="2" t="n">
         <v>7018145</v>
       </c>
-      <c r="C191" s="4" t="inlineStr"/>
-      <c r="D191" s="4" t="inlineStr"/>
-      <c r="E191" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F191" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>WP6610456</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Board - WP6610456</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 7018145; three pages</t>
         </is>
       </c>
     </row>
@@ -4869,24 +5061,24 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="4" t="inlineStr">
+      <c r="A199" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B199" s="4" t="n">
+      <c r="B199" s="3" t="n">
         <v>12329076</v>
       </c>
-      <c r="C199" s="4" t="inlineStr"/>
-      <c r="D199" s="4" t="inlineStr"/>
-      <c r="E199" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F199" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C199" s="3" t="inlineStr"/>
+      <c r="D199" s="3" t="inlineStr"/>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -5023,90 +5215,106 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="4" t="inlineStr">
+      <c r="A206" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B206" s="4" t="n">
+      <c r="B206" s="2" t="n">
         <v>11436692</v>
       </c>
-      <c r="C206" s="4" t="inlineStr"/>
-      <c r="D206" s="4" t="inlineStr"/>
-      <c r="E206" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F206" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>W11122557</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Board - W11122557</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 11436692; single page</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="4" t="inlineStr">
+      <c r="A207" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B207" s="4" t="n">
+      <c r="B207" s="3" t="n">
         <v>11436685</v>
       </c>
-      <c r="C207" s="4" t="inlineStr"/>
-      <c r="D207" s="4" t="inlineStr"/>
-      <c r="E207" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F207" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C207" s="3" t="inlineStr"/>
+      <c r="D207" s="3" t="inlineStr"/>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="4" t="inlineStr">
+      <c r="A208" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B208" s="4" t="n">
+      <c r="B208" s="3" t="n">
         <v>11436676</v>
       </c>
-      <c r="C208" s="4" t="inlineStr"/>
-      <c r="D208" s="4" t="inlineStr"/>
-      <c r="E208" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F208" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C208" s="3" t="inlineStr"/>
+      <c r="D208" s="3" t="inlineStr"/>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="4" t="inlineStr">
+      <c r="A209" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B209" s="4" t="n">
+      <c r="B209" s="3" t="n">
         <v>11436503</v>
       </c>
-      <c r="C209" s="4" t="inlineStr"/>
-      <c r="D209" s="4" t="inlineStr"/>
-      <c r="E209" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F209" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>W11113848</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Board - W11113848</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 11436503; only a repair Q&amp;A page names it, type not confirmed</t>
         </is>
       </c>
     </row>
@@ -5221,288 +5429,304 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="4" t="inlineStr">
+      <c r="A215" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B215" s="4" t="n">
+      <c r="B215" s="3" t="n">
         <v>12925362</v>
       </c>
-      <c r="C215" s="4" t="inlineStr"/>
-      <c r="D215" s="4" t="inlineStr"/>
-      <c r="E215" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F215" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C215" s="3" t="inlineStr"/>
+      <c r="D215" s="3" t="inlineStr"/>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="4" t="inlineStr">
+      <c r="A216" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B216" s="4" t="n">
+      <c r="B216" s="2" t="n">
         <v>9657916</v>
       </c>
-      <c r="C216" s="4" t="inlineStr"/>
-      <c r="D216" s="4" t="inlineStr"/>
-      <c r="E216" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F216" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>910831</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Griddle Kit - 910831</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9657916; replaces 910734</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="4" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B217" s="4" t="n">
+      <c r="B217" s="2" t="n">
         <v>9657362</v>
       </c>
-      <c r="C217" s="4" t="inlineStr"/>
-      <c r="D217" s="4" t="inlineStr"/>
-      <c r="E217" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F217" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>409050</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Logic Card - 409050</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9657362; single page</t>
         </is>
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="4" t="inlineStr">
+      <c r="A218" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B218" s="4" t="n">
+      <c r="B218" s="3" t="n">
         <v>9657361</v>
       </c>
-      <c r="C218" s="4" t="inlineStr"/>
-      <c r="D218" s="4" t="inlineStr"/>
-      <c r="E218" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F218" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C218" s="3" t="inlineStr"/>
+      <c r="D218" s="3" t="inlineStr"/>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="4" t="inlineStr">
+      <c r="A219" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B219" s="4" t="n">
+      <c r="B219" s="3" t="n">
         <v>9656609</v>
       </c>
-      <c r="C219" s="4" t="inlineStr"/>
-      <c r="D219" s="4" t="inlineStr"/>
-      <c r="E219" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F219" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C219" s="3" t="inlineStr"/>
+      <c r="D219" s="3" t="inlineStr"/>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="4" t="inlineStr">
+      <c r="A220" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B220" s="4" t="n">
+      <c r="B220" s="3" t="n">
         <v>9656674</v>
       </c>
-      <c r="C220" s="4" t="inlineStr"/>
-      <c r="D220" s="4" t="inlineStr"/>
-      <c r="E220" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F220" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C220" s="3" t="inlineStr"/>
+      <c r="D220" s="3" t="inlineStr"/>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="4" t="inlineStr">
+      <c r="A221" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B221" s="4" t="n">
+      <c r="B221" s="3" t="n">
         <v>9656567</v>
       </c>
-      <c r="C221" s="4" t="inlineStr"/>
-      <c r="D221" s="4" t="inlineStr"/>
-      <c r="E221" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F221" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C221" s="3" t="inlineStr"/>
+      <c r="D221" s="3" t="inlineStr"/>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="4" t="inlineStr">
+      <c r="A222" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B222" s="4" t="n">
+      <c r="B222" s="3" t="n">
         <v>9656550</v>
       </c>
-      <c r="C222" s="4" t="inlineStr"/>
-      <c r="D222" s="4" t="inlineStr"/>
-      <c r="E222" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F222" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C222" s="3" t="inlineStr"/>
+      <c r="D222" s="3" t="inlineStr"/>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="4" t="inlineStr">
+      <c r="A223" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B223" s="4" t="n">
+      <c r="B223" s="3" t="n">
         <v>12319081</v>
       </c>
-      <c r="C223" s="4" t="inlineStr"/>
-      <c r="D223" s="4" t="inlineStr"/>
-      <c r="E223" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F223" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C223" s="3" t="inlineStr"/>
+      <c r="D223" s="3" t="inlineStr"/>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="4" t="inlineStr">
+      <c r="A224" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B224" s="4" t="n">
+      <c r="B224" s="3" t="n">
         <v>12319074</v>
       </c>
-      <c r="C224" s="4" t="inlineStr"/>
-      <c r="D224" s="4" t="inlineStr"/>
-      <c r="E224" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F224" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C224" s="3" t="inlineStr"/>
+      <c r="D224" s="3" t="inlineStr"/>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="4" t="inlineStr">
+      <c r="A225" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B225" s="4" t="n">
+      <c r="B225" s="3" t="n">
         <v>12319073</v>
       </c>
-      <c r="C225" s="4" t="inlineStr"/>
-      <c r="D225" s="4" t="inlineStr"/>
-      <c r="E225" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F225" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C225" s="3" t="inlineStr"/>
+      <c r="D225" s="3" t="inlineStr"/>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="4" t="inlineStr">
+      <c r="A226" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B226" s="4" t="n">
+      <c r="B226" s="3" t="n">
         <v>12319099</v>
       </c>
-      <c r="C226" s="4" t="inlineStr"/>
-      <c r="D226" s="4" t="inlineStr"/>
-      <c r="E226" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F226" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C226" s="3" t="inlineStr"/>
+      <c r="D226" s="3" t="inlineStr"/>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="4" t="inlineStr">
+      <c r="A227" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B227" s="4" t="n">
+      <c r="B227" s="3" t="n">
         <v>12319087</v>
       </c>
-      <c r="C227" s="4" t="inlineStr"/>
-      <c r="D227" s="4" t="inlineStr"/>
-      <c r="E227" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F227" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C227" s="3" t="inlineStr"/>
+      <c r="D227" s="3" t="inlineStr"/>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Range Collection H1 tags: mark Bosch/Blomberg lookups
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -5951,222 +5951,226 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="4" t="inlineStr">
+      <c r="A238" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B238" s="4" t="n">
+      <c r="B238" s="3" t="n">
         <v>12925667</v>
       </c>
-      <c r="C238" s="4" t="inlineStr"/>
-      <c r="D238" s="4" t="inlineStr"/>
-      <c r="E238" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F238" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C238" s="3" t="inlineStr"/>
+      <c r="D238" s="3" t="inlineStr"/>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="4" t="inlineStr">
+      <c r="A239" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B239" s="4" t="n">
+      <c r="B239" s="3" t="n">
         <v>12499168</v>
       </c>
-      <c r="C239" s="4" t="inlineStr"/>
-      <c r="D239" s="4" t="inlineStr"/>
-      <c r="E239" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F239" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C239" s="3" t="inlineStr"/>
+      <c r="D239" s="3" t="inlineStr"/>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="4" t="inlineStr">
+      <c r="A240" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B240" s="4" t="n">
+      <c r="B240" s="3" t="n">
         <v>12488483</v>
       </c>
-      <c r="C240" s="4" t="inlineStr"/>
-      <c r="D240" s="4" t="inlineStr"/>
-      <c r="E240" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F240" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C240" s="3" t="inlineStr"/>
+      <c r="D240" s="3" t="inlineStr"/>
+      <c r="E240" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F240" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="4" t="inlineStr">
+      <c r="A241" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B241" s="4" t="n">
+      <c r="B241" s="3" t="n">
         <v>12709500</v>
       </c>
-      <c r="C241" s="4" t="inlineStr"/>
-      <c r="D241" s="4" t="inlineStr"/>
-      <c r="E241" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F241" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C241" s="3" t="inlineStr"/>
+      <c r="D241" s="3" t="inlineStr"/>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="4" t="inlineStr">
+      <c r="A242" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B242" s="4" t="n">
+      <c r="B242" s="3" t="n">
         <v>11829909</v>
       </c>
-      <c r="C242" s="4" t="inlineStr"/>
-      <c r="D242" s="4" t="inlineStr"/>
-      <c r="E242" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F242" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C242" s="3" t="inlineStr"/>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blomberg Range Gas Solenoid &amp; Regulator Assembly - </t>
+        </is>
+      </c>
+      <c r="E242" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="inlineStr">
+        <is>
+          <t>Only a forum thread links it to an Encompass listing for a Beko/Blomberg gas range; manufacturer part number not found</t>
         </is>
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="4" t="inlineStr">
+      <c r="A243" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B243" s="4" t="n">
+      <c r="B243" s="3" t="n">
         <v>11053978</v>
       </c>
-      <c r="C243" s="4" t="inlineStr"/>
-      <c r="D243" s="4" t="inlineStr"/>
-      <c r="E243" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F243" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C243" s="3" t="inlineStr"/>
+      <c r="D243" s="3" t="inlineStr"/>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="4" t="inlineStr">
+      <c r="A244" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B244" s="4" t="n">
+      <c r="B244" s="3" t="n">
         <v>11598732</v>
       </c>
-      <c r="C244" s="4" t="inlineStr"/>
-      <c r="D244" s="4" t="inlineStr"/>
-      <c r="E244" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F244" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C244" s="3" t="inlineStr"/>
+      <c r="D244" s="3" t="inlineStr"/>
+      <c r="E244" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F244" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="4" t="inlineStr">
+      <c r="A245" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B245" s="4" t="n">
+      <c r="B245" s="3" t="n">
         <v>12282197</v>
       </c>
-      <c r="C245" s="4" t="inlineStr"/>
-      <c r="D245" s="4" t="inlineStr"/>
-      <c r="E245" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F245" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C245" s="3" t="inlineStr"/>
+      <c r="D245" s="3" t="inlineStr"/>
+      <c r="E245" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F245" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="4" t="inlineStr">
+      <c r="A246" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B246" s="4" t="n">
+      <c r="B246" s="3" t="n">
         <v>11598731</v>
       </c>
-      <c r="C246" s="4" t="inlineStr"/>
-      <c r="D246" s="4" t="inlineStr"/>
-      <c r="E246" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F246" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C246" s="3" t="inlineStr"/>
+      <c r="D246" s="3" t="inlineStr"/>
+      <c r="E246" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F246" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="4" t="inlineStr">
+      <c r="A247" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B247" s="4" t="n">
+      <c r="B247" s="3" t="n">
         <v>12444669</v>
       </c>
-      <c r="C247" s="4" t="inlineStr"/>
-      <c r="D247" s="4" t="inlineStr"/>
-      <c r="E247" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F247" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C247" s="3" t="inlineStr"/>
+      <c r="D247" s="3" t="inlineStr"/>
+      <c r="E247" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F247" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Range Collection H1 tags: Frigidaire/GE lookups
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -6241,90 +6241,90 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="4" t="inlineStr">
+      <c r="A251" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B251" s="4" t="n">
+      <c r="B251" s="3" t="n">
         <v>6953935</v>
       </c>
-      <c r="C251" s="4" t="inlineStr"/>
-      <c r="D251" s="4" t="inlineStr"/>
-      <c r="E251" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F251" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C251" s="3" t="inlineStr"/>
+      <c r="D251" s="3" t="inlineStr"/>
+      <c r="E251" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F251" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="4" t="inlineStr">
+      <c r="A252" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B252" s="4" t="n">
+      <c r="B252" s="3" t="n">
         <v>11580852</v>
       </c>
-      <c r="C252" s="4" t="inlineStr"/>
-      <c r="D252" s="4" t="inlineStr"/>
-      <c r="E252" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F252" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C252" s="3" t="inlineStr"/>
+      <c r="D252" s="3" t="inlineStr"/>
+      <c r="E252" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F252" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="4" t="inlineStr">
+      <c r="A253" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B253" s="4" t="n">
+      <c r="B253" s="3" t="n">
         <v>11577484</v>
       </c>
-      <c r="C253" s="4" t="inlineStr"/>
-      <c r="D253" s="4" t="inlineStr"/>
-      <c r="E253" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F253" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C253" s="3" t="inlineStr"/>
+      <c r="D253" s="3" t="inlineStr"/>
+      <c r="E253" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F253" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="4" t="inlineStr">
+      <c r="A254" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B254" s="4" t="n">
+      <c r="B254" s="3" t="n">
         <v>10074064</v>
       </c>
-      <c r="C254" s="4" t="inlineStr"/>
-      <c r="D254" s="4" t="inlineStr"/>
-      <c r="E254" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F254" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C254" s="3" t="inlineStr"/>
+      <c r="D254" s="3" t="inlineStr"/>
+      <c r="E254" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F254" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6351,134 +6351,142 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="4" t="inlineStr">
+      <c r="A256" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B256" s="4" t="n">
+      <c r="B256" s="3" t="n">
         <v>10168871</v>
       </c>
-      <c r="C256" s="4" t="inlineStr"/>
-      <c r="D256" s="4" t="inlineStr"/>
-      <c r="E256" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F256" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C256" s="3" t="inlineStr"/>
+      <c r="D256" s="3" t="inlineStr"/>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F256" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="4" t="inlineStr">
+      <c r="A257" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B257" s="4" t="n">
+      <c r="B257" s="3" t="n">
         <v>10168894</v>
       </c>
-      <c r="C257" s="4" t="inlineStr"/>
-      <c r="D257" s="4" t="inlineStr"/>
-      <c r="E257" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F257" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C257" s="3" t="inlineStr"/>
+      <c r="D257" s="3" t="inlineStr"/>
+      <c r="E257" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F257" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="4" t="inlineStr">
+      <c r="A258" s="2" t="inlineStr">
         <is>
           <t>Fisher &amp; Paykel</t>
         </is>
       </c>
-      <c r="B258" s="4" t="n">
+      <c r="B258" s="2" t="n">
         <v>10387982</v>
       </c>
-      <c r="C258" s="4" t="inlineStr"/>
-      <c r="D258" s="4" t="inlineStr"/>
-      <c r="E258" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F258" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>210782P</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>Fisher &amp; Paykel Range Dual Thermal Gas Valve - 210782P</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 10387982; single page</t>
         </is>
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="4" t="inlineStr">
+      <c r="A259" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B259" s="4" t="n">
+      <c r="B259" s="3" t="n">
         <v>10838321</v>
       </c>
-      <c r="C259" s="4" t="inlineStr"/>
-      <c r="D259" s="4" t="inlineStr"/>
-      <c r="E259" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F259" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C259" s="3" t="inlineStr"/>
+      <c r="D259" s="3" t="inlineStr"/>
+      <c r="E259" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F259" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="4" t="inlineStr">
+      <c r="A260" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B260" s="4" t="n">
+      <c r="B260" s="3" t="n">
         <v>10847437</v>
       </c>
-      <c r="C260" s="4" t="inlineStr"/>
-      <c r="D260" s="4" t="inlineStr"/>
-      <c r="E260" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F260" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C260" s="3" t="inlineStr"/>
+      <c r="D260" s="3" t="inlineStr"/>
+      <c r="E260" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F260" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="4" t="inlineStr">
+      <c r="A261" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B261" s="4" t="n">
+      <c r="B261" s="3" t="n">
         <v>10868484</v>
       </c>
-      <c r="C261" s="4" t="inlineStr"/>
-      <c r="D261" s="4" t="inlineStr"/>
-      <c r="E261" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F261" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C261" s="3" t="inlineStr"/>
+      <c r="D261" s="3" t="inlineStr"/>
+      <c r="E261" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F261" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10047,24 +10055,32 @@
       </c>
     </row>
     <row r="424">
-      <c r="A424" s="4" t="inlineStr">
+      <c r="A424" s="2" t="inlineStr">
         <is>
           <t>Fisher &amp; Paykel</t>
         </is>
       </c>
-      <c r="B424" s="4" t="n">
+      <c r="B424" s="2" t="n">
         <v>10387982</v>
       </c>
-      <c r="C424" s="4" t="inlineStr"/>
-      <c r="D424" s="4" t="inlineStr"/>
-      <c r="E424" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F424" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>210782P</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>Fisher &amp; Paykel Range Dual Thermal Gas Valve - 210782P</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 10387982; single page</t>
         </is>
       </c>
     </row>
@@ -10531,24 +10547,24 @@
       </c>
     </row>
     <row r="446">
-      <c r="A446" s="4" t="inlineStr">
+      <c r="A446" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B446" s="4" t="n">
+      <c r="B446" s="3" t="n">
         <v>6953935</v>
       </c>
-      <c r="C446" s="4" t="inlineStr"/>
-      <c r="D446" s="4" t="inlineStr"/>
-      <c r="E446" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F446" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C446" s="3" t="inlineStr"/>
+      <c r="D446" s="3" t="inlineStr"/>
+      <c r="E446" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F446" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10575,24 +10591,24 @@
       </c>
     </row>
     <row r="448">
-      <c r="A448" s="4" t="inlineStr">
+      <c r="A448" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B448" s="4" t="n">
+      <c r="B448" s="3" t="n">
         <v>10168871</v>
       </c>
-      <c r="C448" s="4" t="inlineStr"/>
-      <c r="D448" s="4" t="inlineStr"/>
-      <c r="E448" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F448" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C448" s="3" t="inlineStr"/>
+      <c r="D448" s="3" t="inlineStr"/>
+      <c r="E448" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F448" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10619,24 +10635,24 @@
       </c>
     </row>
     <row r="450">
-      <c r="A450" s="4" t="inlineStr">
+      <c r="A450" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B450" s="4" t="n">
+      <c r="B450" s="3" t="n">
         <v>11577484</v>
       </c>
-      <c r="C450" s="4" t="inlineStr"/>
-      <c r="D450" s="4" t="inlineStr"/>
-      <c r="E450" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F450" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C450" s="3" t="inlineStr"/>
+      <c r="D450" s="3" t="inlineStr"/>
+      <c r="E450" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F450" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10817,46 +10833,46 @@
       </c>
     </row>
     <row r="459">
-      <c r="A459" s="4" t="inlineStr">
+      <c r="A459" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B459" s="4" t="n">
+      <c r="B459" s="3" t="n">
         <v>11580852</v>
       </c>
-      <c r="C459" s="4" t="inlineStr"/>
-      <c r="D459" s="4" t="inlineStr"/>
-      <c r="E459" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F459" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C459" s="3" t="inlineStr"/>
+      <c r="D459" s="3" t="inlineStr"/>
+      <c r="E459" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F459" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="460">
-      <c r="A460" s="4" t="inlineStr">
+      <c r="A460" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B460" s="4" t="n">
+      <c r="B460" s="3" t="n">
         <v>10868484</v>
       </c>
-      <c r="C460" s="4" t="inlineStr"/>
-      <c r="D460" s="4" t="inlineStr"/>
-      <c r="E460" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F460" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C460" s="3" t="inlineStr"/>
+      <c r="D460" s="3" t="inlineStr"/>
+      <c r="E460" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F460" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10905,24 +10921,24 @@
       </c>
     </row>
     <row r="463">
-      <c r="A463" s="4" t="inlineStr">
+      <c r="A463" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B463" s="4" t="n">
+      <c r="B463" s="3" t="n">
         <v>10847437</v>
       </c>
-      <c r="C463" s="4" t="inlineStr"/>
-      <c r="D463" s="4" t="inlineStr"/>
-      <c r="E463" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F463" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C463" s="3" t="inlineStr"/>
+      <c r="D463" s="3" t="inlineStr"/>
+      <c r="E463" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F463" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -11059,24 +11075,24 @@
       </c>
     </row>
     <row r="470">
-      <c r="A470" s="4" t="inlineStr">
+      <c r="A470" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B470" s="4" t="n">
+      <c r="B470" s="3" t="n">
         <v>10074064</v>
       </c>
-      <c r="C470" s="4" t="inlineStr"/>
-      <c r="D470" s="4" t="inlineStr"/>
-      <c r="E470" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F470" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C470" s="3" t="inlineStr"/>
+      <c r="D470" s="3" t="inlineStr"/>
+      <c r="E470" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F470" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Range collection H1 tags: add more Encompass-resolved titles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -5731,222 +5731,222 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="4" t="inlineStr">
+      <c r="A228" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B228" s="4" t="n">
+      <c r="B228" s="3" t="n">
         <v>12319089</v>
       </c>
-      <c r="C228" s="4" t="inlineStr"/>
-      <c r="D228" s="4" t="inlineStr"/>
-      <c r="E228" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F228" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C228" s="3" t="inlineStr"/>
+      <c r="D228" s="3" t="inlineStr"/>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="4" t="inlineStr">
+      <c r="A229" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B229" s="4" t="n">
+      <c r="B229" s="3" t="n">
         <v>11584933</v>
       </c>
-      <c r="C229" s="4" t="inlineStr"/>
-      <c r="D229" s="4" t="inlineStr"/>
-      <c r="E229" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F229" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C229" s="3" t="inlineStr"/>
+      <c r="D229" s="3" t="inlineStr"/>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="4" t="inlineStr">
+      <c r="A230" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B230" s="4" t="n">
+      <c r="B230" s="3" t="n">
         <v>11584913</v>
       </c>
-      <c r="C230" s="4" t="inlineStr"/>
-      <c r="D230" s="4" t="inlineStr"/>
-      <c r="E230" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F230" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C230" s="3" t="inlineStr"/>
+      <c r="D230" s="3" t="inlineStr"/>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="4" t="inlineStr">
+      <c r="A231" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B231" s="4" t="n">
+      <c r="B231" s="3" t="n">
         <v>11584931</v>
       </c>
-      <c r="C231" s="4" t="inlineStr"/>
-      <c r="D231" s="4" t="inlineStr"/>
-      <c r="E231" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F231" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C231" s="3" t="inlineStr"/>
+      <c r="D231" s="3" t="inlineStr"/>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="4" t="inlineStr">
+      <c r="A232" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B232" s="4" t="n">
+      <c r="B232" s="3" t="n">
         <v>11584932</v>
       </c>
-      <c r="C232" s="4" t="inlineStr"/>
-      <c r="D232" s="4" t="inlineStr"/>
-      <c r="E232" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F232" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C232" s="3" t="inlineStr"/>
+      <c r="D232" s="3" t="inlineStr"/>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="4" t="inlineStr">
+      <c r="A233" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B233" s="4" t="n">
+      <c r="B233" s="3" t="n">
         <v>10681415</v>
       </c>
-      <c r="C233" s="4" t="inlineStr"/>
-      <c r="D233" s="4" t="inlineStr"/>
-      <c r="E233" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F233" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C233" s="3" t="inlineStr"/>
+      <c r="D233" s="3" t="inlineStr"/>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="4" t="inlineStr">
+      <c r="A234" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B234" s="4" t="n">
+      <c r="B234" s="3" t="n">
         <v>10178316</v>
       </c>
-      <c r="C234" s="4" t="inlineStr"/>
-      <c r="D234" s="4" t="inlineStr"/>
-      <c r="E234" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F234" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C234" s="3" t="inlineStr"/>
+      <c r="D234" s="3" t="inlineStr"/>
+      <c r="E234" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F234" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="4" t="inlineStr">
+      <c r="A235" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B235" s="4" t="n">
+      <c r="B235" s="3" t="n">
         <v>12710552</v>
       </c>
-      <c r="C235" s="4" t="inlineStr"/>
-      <c r="D235" s="4" t="inlineStr"/>
-      <c r="E235" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F235" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C235" s="3" t="inlineStr"/>
+      <c r="D235" s="3" t="inlineStr"/>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="4" t="inlineStr">
+      <c r="A236" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B236" s="4" t="n">
+      <c r="B236" s="3" t="n">
         <v>12320902</v>
       </c>
-      <c r="C236" s="4" t="inlineStr"/>
-      <c r="D236" s="4" t="inlineStr"/>
-      <c r="E236" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F236" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C236" s="3" t="inlineStr"/>
+      <c r="D236" s="3" t="inlineStr"/>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="4" t="inlineStr">
+      <c r="A237" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B237" s="4" t="n">
+      <c r="B237" s="3" t="n">
         <v>12320894</v>
       </c>
-      <c r="C237" s="4" t="inlineStr"/>
-      <c r="D237" s="4" t="inlineStr"/>
-      <c r="E237" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F237" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C237" s="3" t="inlineStr"/>
+      <c r="D237" s="3" t="inlineStr"/>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6175,68 +6175,68 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="4" t="inlineStr">
+      <c r="A248" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B248" s="4" t="n">
+      <c r="B248" s="3" t="n">
         <v>12499480</v>
       </c>
-      <c r="C248" s="4" t="inlineStr"/>
-      <c r="D248" s="4" t="inlineStr"/>
-      <c r="E248" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F248" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C248" s="3" t="inlineStr"/>
+      <c r="D248" s="3" t="inlineStr"/>
+      <c r="E248" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F248" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="4" t="inlineStr">
+      <c r="A249" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B249" s="4" t="n">
+      <c r="B249" s="3" t="n">
         <v>11597884</v>
       </c>
-      <c r="C249" s="4" t="inlineStr"/>
-      <c r="D249" s="4" t="inlineStr"/>
-      <c r="E249" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F249" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C249" s="3" t="inlineStr"/>
+      <c r="D249" s="3" t="inlineStr"/>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="4" t="inlineStr">
+      <c r="A250" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B250" s="4" t="n">
+      <c r="B250" s="3" t="n">
         <v>12469969</v>
       </c>
-      <c r="C250" s="4" t="inlineStr"/>
-      <c r="D250" s="4" t="inlineStr"/>
-      <c r="E250" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F250" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C250" s="3" t="inlineStr"/>
+      <c r="D250" s="3" t="inlineStr"/>
+      <c r="E250" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F250" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6329,24 +6329,24 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="4" t="inlineStr">
+      <c r="A255" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B255" s="4" t="n">
+      <c r="B255" s="3" t="n">
         <v>10130655</v>
       </c>
-      <c r="C255" s="4" t="inlineStr"/>
-      <c r="D255" s="4" t="inlineStr"/>
-      <c r="E255" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F255" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C255" s="3" t="inlineStr"/>
+      <c r="D255" s="3" t="inlineStr"/>
+      <c r="E255" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F255" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6491,46 +6491,54 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="4" t="inlineStr">
+      <c r="A262" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B262" s="4" t="n">
+      <c r="B262" s="3" t="n">
         <v>10878840</v>
       </c>
-      <c r="C262" s="4" t="inlineStr"/>
-      <c r="D262" s="4" t="inlineStr"/>
-      <c r="E262" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F262" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C262" s="3" t="inlineStr"/>
+      <c r="D262" s="3" t="inlineStr"/>
+      <c r="E262" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F262" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="4" t="inlineStr">
+      <c r="A263" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B263" s="4" t="n">
+      <c r="B263" s="3" t="n">
         <v>10879182</v>
       </c>
-      <c r="C263" s="4" t="inlineStr"/>
-      <c r="D263" s="4" t="inlineStr"/>
-      <c r="E263" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F263" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>807038640</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>Electrolux Cooktop SmoothTop Glass &amp; Steel Assembly - 807038640</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F263" s="3" t="inlineStr">
+        <is>
+          <t>Listing shows 10879182 as base part for model 807038640; single seller page</t>
         </is>
       </c>
     </row>
@@ -6623,24 +6631,24 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="4" t="inlineStr">
+      <c r="A268" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B268" s="4" t="n">
+      <c r="B268" s="3" t="n">
         <v>11578315</v>
       </c>
-      <c r="C268" s="4" t="inlineStr"/>
-      <c r="D268" s="4" t="inlineStr"/>
-      <c r="E268" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F268" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C268" s="3" t="inlineStr"/>
+      <c r="D268" s="3" t="inlineStr"/>
+      <c r="E268" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F268" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6799,24 +6807,24 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" s="4" t="inlineStr">
+      <c r="A276" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B276" s="4" t="n">
+      <c r="B276" s="3" t="n">
         <v>11654521</v>
       </c>
-      <c r="C276" s="4" t="inlineStr"/>
-      <c r="D276" s="4" t="inlineStr"/>
-      <c r="E276" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F276" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C276" s="3" t="inlineStr"/>
+      <c r="D276" s="3" t="inlineStr"/>
+      <c r="E276" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F276" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6843,24 +6851,32 @@
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="4" t="inlineStr">
+      <c r="A278" s="2" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B278" s="4" t="n">
+      <c r="B278" s="2" t="n">
         <v>12427085</v>
       </c>
-      <c r="C278" s="4" t="inlineStr"/>
-      <c r="D278" s="4" t="inlineStr"/>
-      <c r="E278" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F278" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>WB27X33137</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>GE Range Oven Control &amp; Overlay Assembly - WB27X33137</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 12427085; single page</t>
         </is>
       </c>
     </row>
@@ -6931,46 +6947,54 @@
       </c>
     </row>
     <row r="282">
-      <c r="A282" s="4" t="inlineStr">
+      <c r="A282" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B282" s="4" t="n">
+      <c r="B282" s="3" t="n">
         <v>12619548</v>
       </c>
-      <c r="C282" s="4" t="inlineStr"/>
-      <c r="D282" s="4" t="inlineStr"/>
-      <c r="E282" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F282" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C282" s="3" t="inlineStr"/>
+      <c r="D282" s="3" t="inlineStr"/>
+      <c r="E282" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F282" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="283">
-      <c r="A283" s="4" t="inlineStr">
+      <c r="A283" s="2" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B283" s="4" t="n">
+      <c r="B283" s="2" t="n">
         <v>12632407</v>
       </c>
-      <c r="C283" s="4" t="inlineStr"/>
-      <c r="D283" s="4" t="inlineStr"/>
-      <c r="E283" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F283" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>WB27X39826</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>GE Range Stainless UI LCD Control Panel - WB27X39826</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 12632407; single page</t>
         </is>
       </c>
     </row>
@@ -7041,860 +7065,916 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="4" t="inlineStr">
+      <c r="A287" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B287" s="4" t="n">
+      <c r="B287" s="3" t="n">
         <v>6862572</v>
       </c>
-      <c r="C287" s="4" t="inlineStr"/>
-      <c r="D287" s="4" t="inlineStr"/>
-      <c r="E287" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F287" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C287" s="3" t="inlineStr"/>
+      <c r="D287" s="3" t="inlineStr"/>
+      <c r="E287" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F287" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="4" t="inlineStr">
+      <c r="A288" s="2" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B288" s="4" t="n">
+      <c r="B288" s="2" t="n">
         <v>6874796</v>
       </c>
-      <c r="C288" s="4" t="inlineStr"/>
-      <c r="D288" s="4" t="inlineStr"/>
-      <c r="E288" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F288" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>WB57K5</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>GE Range Glass Door - WB57K5</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 6874796; three Encompass pages</t>
         </is>
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="4" t="inlineStr">
+      <c r="A289" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B289" s="4" t="n">
+      <c r="B289" s="3" t="n">
         <v>6947174</v>
       </c>
-      <c r="C289" s="4" t="inlineStr"/>
-      <c r="D289" s="4" t="inlineStr"/>
-      <c r="E289" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F289" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C289" s="3" t="inlineStr"/>
+      <c r="D289" s="3" t="inlineStr"/>
+      <c r="E289" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F289" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="4" t="inlineStr">
+      <c r="A290" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B290" s="4" t="n">
+      <c r="B290" s="3" t="n">
         <v>6953830</v>
       </c>
-      <c r="C290" s="4" t="inlineStr"/>
-      <c r="D290" s="4" t="inlineStr"/>
-      <c r="E290" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F290" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C290" s="3" t="inlineStr"/>
+      <c r="D290" s="3" t="inlineStr"/>
+      <c r="E290" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F290" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="4" t="inlineStr">
+      <c r="A291" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B291" s="4" t="n">
+      <c r="B291" s="3" t="n">
         <v>6947945</v>
       </c>
-      <c r="C291" s="4" t="inlineStr"/>
-      <c r="D291" s="4" t="inlineStr"/>
-      <c r="E291" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F291" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C291" s="3" t="inlineStr"/>
+      <c r="D291" s="3" t="inlineStr"/>
+      <c r="E291" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F291" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="4" t="inlineStr">
+      <c r="A292" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B292" s="4" t="n">
+      <c r="B292" s="3" t="n">
         <v>6948923</v>
       </c>
-      <c r="C292" s="4" t="inlineStr"/>
-      <c r="D292" s="4" t="inlineStr"/>
-      <c r="E292" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F292" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C292" s="3" t="inlineStr"/>
+      <c r="D292" s="3" t="inlineStr"/>
+      <c r="E292" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F292" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="4" t="inlineStr">
+      <c r="A293" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B293" s="4" t="n">
+      <c r="B293" s="3" t="n">
         <v>8089749</v>
       </c>
-      <c r="C293" s="4" t="inlineStr"/>
-      <c r="D293" s="4" t="inlineStr"/>
-      <c r="E293" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F293" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C293" s="3" t="inlineStr"/>
+      <c r="D293" s="3" t="inlineStr"/>
+      <c r="E293" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F293" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="4" t="inlineStr">
+      <c r="A294" s="2" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B294" s="4" t="n">
+      <c r="B294" s="2" t="n">
         <v>9329006</v>
       </c>
-      <c r="C294" s="4" t="inlineStr"/>
-      <c r="D294" s="4" t="inlineStr"/>
-      <c r="E294" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F294" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>WB27T11076</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>GE Range Keypanel Support Assembly (Black) - WB27T11076</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9329006; two Encompass pages</t>
         </is>
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="4" t="inlineStr">
+      <c r="A295" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B295" s="4" t="n">
+      <c r="B295" s="3" t="n">
         <v>9328045</v>
       </c>
-      <c r="C295" s="4" t="inlineStr"/>
-      <c r="D295" s="4" t="inlineStr"/>
-      <c r="E295" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F295" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C295" s="3" t="inlineStr"/>
+      <c r="D295" s="3" t="inlineStr"/>
+      <c r="E295" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F295" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="4" t="inlineStr">
+      <c r="A296" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B296" s="4" t="n">
+      <c r="B296" s="3" t="n">
         <v>9331494</v>
       </c>
-      <c r="C296" s="4" t="inlineStr"/>
-      <c r="D296" s="4" t="inlineStr"/>
-      <c r="E296" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F296" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C296" s="3" t="inlineStr"/>
+      <c r="D296" s="3" t="inlineStr"/>
+      <c r="E296" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F296" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="4" t="inlineStr">
+      <c r="A297" s="2" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B297" s="4" t="n">
+      <c r="B297" s="2" t="n">
         <v>9328760</v>
       </c>
-      <c r="C297" s="4" t="inlineStr"/>
-      <c r="D297" s="4" t="inlineStr"/>
-      <c r="E297" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F297" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>WB27K10245</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>GE Range Oven Control (T011) - WB27K10245</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr">
+        <is>
+          <t>Encompass listing ID 9328760; three Encompass pages</t>
         </is>
       </c>
     </row>
     <row r="298">
-      <c r="A298" s="4" t="inlineStr">
+      <c r="A298" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B298" s="4" t="n">
+      <c r="B298" s="3" t="n">
         <v>9350706</v>
       </c>
-      <c r="C298" s="4" t="inlineStr"/>
-      <c r="D298" s="4" t="inlineStr"/>
-      <c r="E298" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F298" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C298" s="3" t="inlineStr"/>
+      <c r="D298" s="3" t="inlineStr"/>
+      <c r="E298" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F298" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="4" t="inlineStr">
+      <c r="A299" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B299" s="4" t="n">
+      <c r="B299" s="3" t="n">
         <v>9349281</v>
       </c>
-      <c r="C299" s="4" t="inlineStr"/>
-      <c r="D299" s="4" t="inlineStr"/>
-      <c r="E299" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F299" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C299" s="3" t="inlineStr"/>
+      <c r="D299" s="3" t="inlineStr"/>
+      <c r="E299" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F299" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="4" t="inlineStr">
+      <c r="A300" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B300" s="4" t="n">
+      <c r="B300" s="3" t="n">
         <v>9349682</v>
       </c>
-      <c r="C300" s="4" t="inlineStr"/>
-      <c r="D300" s="4" t="inlineStr"/>
-      <c r="E300" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F300" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C300" s="3" t="inlineStr"/>
+      <c r="D300" s="3" t="inlineStr"/>
+      <c r="E300" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F300" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="4" t="inlineStr">
+      <c r="A301" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B301" s="4" t="n">
+      <c r="B301" s="3" t="n">
         <v>9835037</v>
       </c>
-      <c r="C301" s="4" t="inlineStr"/>
-      <c r="D301" s="4" t="inlineStr"/>
-      <c r="E301" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F301" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C301" s="3" t="inlineStr"/>
+      <c r="D301" s="3" t="inlineStr"/>
+      <c r="E301" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F301" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="4" t="inlineStr">
+      <c r="A302" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B302" s="4" t="n">
+      <c r="B302" s="3" t="n">
         <v>9835005</v>
       </c>
-      <c r="C302" s="4" t="inlineStr"/>
-      <c r="D302" s="4" t="inlineStr"/>
-      <c r="E302" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F302" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C302" s="3" t="inlineStr"/>
+      <c r="D302" s="3" t="inlineStr"/>
+      <c r="E302" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F302" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="4" t="inlineStr">
+      <c r="A303" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B303" s="4" t="n">
+      <c r="B303" s="3" t="n">
         <v>9835061</v>
       </c>
-      <c r="C303" s="4" t="inlineStr"/>
-      <c r="D303" s="4" t="inlineStr"/>
-      <c r="E303" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F303" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C303" s="3" t="inlineStr"/>
+      <c r="D303" s="3" t="inlineStr"/>
+      <c r="E303" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F303" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="4" t="inlineStr">
+      <c r="A304" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B304" s="4" t="n">
+      <c r="B304" s="3" t="n">
         <v>9349282</v>
       </c>
-      <c r="C304" s="4" t="inlineStr"/>
-      <c r="D304" s="4" t="inlineStr"/>
-      <c r="E304" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F304" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C304" s="3" t="inlineStr"/>
+      <c r="D304" s="3" t="inlineStr"/>
+      <c r="E304" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F304" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="4" t="inlineStr">
+      <c r="A305" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B305" s="4" t="n">
+      <c r="B305" s="3" t="n">
         <v>9349296</v>
       </c>
-      <c r="C305" s="4" t="inlineStr"/>
-      <c r="D305" s="4" t="inlineStr"/>
-      <c r="E305" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F305" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C305" s="3" t="inlineStr"/>
+      <c r="D305" s="3" t="inlineStr"/>
+      <c r="E305" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F305" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="4" t="inlineStr">
+      <c r="A306" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B306" s="4" t="n">
+      <c r="B306" s="3" t="n">
         <v>9349191</v>
       </c>
-      <c r="C306" s="4" t="inlineStr"/>
-      <c r="D306" s="4" t="inlineStr"/>
-      <c r="E306" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F306" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C306" s="3" t="inlineStr"/>
+      <c r="D306" s="3" t="inlineStr"/>
+      <c r="E306" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F306" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="4" t="inlineStr">
+      <c r="A307" s="2" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B307" s="4" t="n">
+      <c r="B307" s="2" t="n">
         <v>9349093</v>
       </c>
-      <c r="C307" s="4" t="inlineStr"/>
-      <c r="D307" s="4" t="inlineStr"/>
-      <c r="E307" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F307" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>316443916</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Relay Board - 316443916</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 9349093; fits EW30 range models per listing</t>
         </is>
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="4" t="inlineStr">
+      <c r="A308" s="2" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B308" s="4" t="n">
+      <c r="B308" s="2" t="n">
         <v>9350269</v>
       </c>
-      <c r="C308" s="4" t="inlineStr"/>
-      <c r="D308" s="4" t="inlineStr"/>
-      <c r="E308" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F308" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>316576610</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Electronic Controller (ES630) - 316576610</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 9350269 listed under brand Electrolux; fits EW30 range models per listing</t>
         </is>
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="4" t="inlineStr">
+      <c r="A309" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B309" s="4" t="n">
+      <c r="B309" s="3" t="n">
         <v>9349290</v>
       </c>
-      <c r="C309" s="4" t="inlineStr"/>
-      <c r="D309" s="4" t="inlineStr"/>
-      <c r="E309" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F309" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C309" s="3" t="inlineStr"/>
+      <c r="D309" s="3" t="inlineStr"/>
+      <c r="E309" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F309" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="4" t="inlineStr">
+      <c r="A310" s="2" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B310" s="4" t="n">
+      <c r="B310" s="2" t="n">
         <v>9350077</v>
       </c>
-      <c r="C310" s="4" t="inlineStr"/>
-      <c r="D310" s="4" t="inlineStr"/>
-      <c r="E310" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F310" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>316560118</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Electronic Controller (ES540) - 316560118</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 9350077 listed under brand Electrolux; fits FGGF-series ranges per listing</t>
         </is>
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="4" t="inlineStr">
+      <c r="A311" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B311" s="4" t="n">
+      <c r="B311" s="3" t="n">
         <v>9835004</v>
       </c>
-      <c r="C311" s="4" t="inlineStr"/>
-      <c r="D311" s="4" t="inlineStr"/>
-      <c r="E311" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F311" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C311" s="3" t="inlineStr"/>
+      <c r="D311" s="3" t="inlineStr"/>
+      <c r="E311" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F311" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="4" t="inlineStr">
+      <c r="A312" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B312" s="4" t="n">
+      <c r="B312" s="3" t="n">
         <v>9835036</v>
       </c>
-      <c r="C312" s="4" t="inlineStr"/>
-      <c r="D312" s="4" t="inlineStr"/>
-      <c r="E312" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F312" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C312" s="3" t="inlineStr"/>
+      <c r="D312" s="3" t="inlineStr"/>
+      <c r="E312" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F312" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="4" t="inlineStr">
+      <c r="A313" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B313" s="4" t="n">
+      <c r="B313" s="3" t="n">
         <v>9835062</v>
       </c>
-      <c r="C313" s="4" t="inlineStr"/>
-      <c r="D313" s="4" t="inlineStr"/>
-      <c r="E313" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F313" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C313" s="3" t="inlineStr"/>
+      <c r="D313" s="3" t="inlineStr"/>
+      <c r="E313" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F313" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="4" t="inlineStr">
+      <c r="A314" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B314" s="4" t="n">
+      <c r="B314" s="3" t="n">
         <v>9349047</v>
       </c>
-      <c r="C314" s="4" t="inlineStr"/>
-      <c r="D314" s="4" t="inlineStr"/>
-      <c r="E314" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F314" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C314" s="3" t="inlineStr"/>
+      <c r="D314" s="3" t="inlineStr"/>
+      <c r="E314" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F314" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="4" t="inlineStr">
+      <c r="A315" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B315" s="4" t="n">
+      <c r="B315" s="3" t="n">
         <v>11654923</v>
       </c>
-      <c r="C315" s="4" t="inlineStr"/>
-      <c r="D315" s="4" t="inlineStr"/>
-      <c r="E315" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F315" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C315" s="3" t="inlineStr"/>
+      <c r="D315" s="3" t="inlineStr"/>
+      <c r="E315" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F315" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="4" t="inlineStr">
+      <c r="A316" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B316" s="4" t="n">
+      <c r="B316" s="3" t="n">
         <v>11578959</v>
       </c>
-      <c r="C316" s="4" t="inlineStr"/>
-      <c r="D316" s="4" t="inlineStr"/>
-      <c r="E316" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F316" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C316" s="3" t="inlineStr"/>
+      <c r="D316" s="3" t="inlineStr"/>
+      <c r="E316" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F316" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="4" t="inlineStr">
+      <c r="A317" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B317" s="4" t="n">
+      <c r="B317" s="3" t="n">
         <v>11579003</v>
       </c>
-      <c r="C317" s="4" t="inlineStr"/>
-      <c r="D317" s="4" t="inlineStr"/>
-      <c r="E317" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F317" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C317" s="3" t="inlineStr"/>
+      <c r="D317" s="3" t="inlineStr"/>
+      <c r="E317" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F317" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="4" t="inlineStr">
+      <c r="A318" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B318" s="4" t="n">
+      <c r="B318" s="3" t="n">
         <v>10848443</v>
       </c>
-      <c r="C318" s="4" t="inlineStr"/>
-      <c r="D318" s="4" t="inlineStr"/>
-      <c r="E318" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F318" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C318" s="3" t="inlineStr"/>
+      <c r="D318" s="3" t="inlineStr"/>
+      <c r="E318" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F318" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="4" t="inlineStr">
+      <c r="A319" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B319" s="4" t="n">
+      <c r="B319" s="3" t="n">
         <v>12432120</v>
       </c>
-      <c r="C319" s="4" t="inlineStr"/>
-      <c r="D319" s="4" t="inlineStr"/>
-      <c r="E319" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F319" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C319" s="3" t="inlineStr"/>
+      <c r="D319" s="3" t="inlineStr"/>
+      <c r="E319" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F319" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="4" t="inlineStr">
+      <c r="A320" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B320" s="4" t="n">
+      <c r="B320" s="3" t="n">
         <v>12537681</v>
       </c>
-      <c r="C320" s="4" t="inlineStr"/>
-      <c r="D320" s="4" t="inlineStr"/>
-      <c r="E320" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F320" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C320" s="3" t="inlineStr"/>
+      <c r="D320" s="3" t="inlineStr"/>
+      <c r="E320" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F320" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="4" t="inlineStr">
+      <c r="A321" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B321" s="4" t="n">
+      <c r="B321" s="3" t="n">
         <v>12616076</v>
       </c>
-      <c r="C321" s="4" t="inlineStr"/>
-      <c r="D321" s="4" t="inlineStr"/>
-      <c r="E321" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F321" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C321" s="3" t="inlineStr"/>
+      <c r="D321" s="3" t="inlineStr"/>
+      <c r="E321" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F321" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="4" t="inlineStr">
+      <c r="A322" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B322" s="4" t="n">
+      <c r="B322" s="3" t="n">
         <v>12616092</v>
       </c>
-      <c r="C322" s="4" t="inlineStr"/>
-      <c r="D322" s="4" t="inlineStr"/>
-      <c r="E322" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F322" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C322" s="3" t="inlineStr"/>
+      <c r="D322" s="3" t="inlineStr"/>
+      <c r="E322" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F322" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="4" t="inlineStr">
+      <c r="A323" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B323" s="4" t="n">
+      <c r="B323" s="3" t="n">
         <v>10848602</v>
       </c>
-      <c r="C323" s="4" t="inlineStr"/>
-      <c r="D323" s="4" t="inlineStr"/>
-      <c r="E323" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F323" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C323" s="3" t="inlineStr">
+        <is>
+          <t>WB24X24087</t>
+        </is>
+      </c>
+      <c r="D323" s="3" t="inlineStr">
+        <is>
+          <t>GE Thermostat - WB24X24087</t>
+        </is>
+      </c>
+      <c r="E323" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F323" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 10848602; listing shows refrigerator (ZDP) models, not a range - appliance type omitted, verify</t>
         </is>
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="4" t="inlineStr">
+      <c r="A324" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B324" s="4" t="n">
+      <c r="B324" s="3" t="n">
         <v>12574883</v>
       </c>
-      <c r="C324" s="4" t="inlineStr"/>
-      <c r="D324" s="4" t="inlineStr"/>
-      <c r="E324" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F324" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C324" s="3" t="inlineStr"/>
+      <c r="D324" s="3" t="inlineStr"/>
+      <c r="E324" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F324" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="4" t="inlineStr">
+      <c r="A325" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B325" s="4" t="n">
+      <c r="B325" s="3" t="n">
         <v>12444096</v>
       </c>
-      <c r="C325" s="4" t="inlineStr"/>
-      <c r="D325" s="4" t="inlineStr"/>
-      <c r="E325" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F325" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C325" s="3" t="inlineStr"/>
+      <c r="D325" s="3" t="inlineStr"/>
+      <c r="E325" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F325" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -7921,112 +8001,128 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="4" t="inlineStr">
+      <c r="A327" s="2" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B327" s="4" t="n">
+      <c r="B327" s="2" t="n">
         <v>11578327</v>
       </c>
-      <c r="C327" s="4" t="inlineStr"/>
-      <c r="D327" s="4" t="inlineStr"/>
-      <c r="E327" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F327" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>5304511258</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>Frigidaire Range SmoothTop Glass Assembly (Black) - 5304511258</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 11578327 listed under brand Electrolux</t>
         </is>
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="4" t="inlineStr">
+      <c r="A328" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B328" s="4" t="n">
+      <c r="B328" s="3" t="n">
         <v>12524352</v>
       </c>
-      <c r="C328" s="4" t="inlineStr"/>
-      <c r="D328" s="4" t="inlineStr"/>
-      <c r="E328" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F328" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C328" s="3" t="inlineStr"/>
+      <c r="D328" s="3" t="inlineStr"/>
+      <c r="E328" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F328" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="4" t="inlineStr">
+      <c r="A329" s="2" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B329" s="4" t="n">
+      <c r="B329" s="2" t="n">
         <v>12732070</v>
       </c>
-      <c r="C329" s="4" t="inlineStr"/>
-      <c r="D329" s="4" t="inlineStr"/>
-      <c r="E329" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F329" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>5304527384</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Induction Power Generator Board - 5304527384</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 12732070; fits GCRI/FGIH induction range models per listing</t>
         </is>
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="4" t="inlineStr">
+      <c r="A330" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B330" s="4" t="n">
+      <c r="B330" s="3" t="n">
         <v>12444423</v>
       </c>
-      <c r="C330" s="4" t="inlineStr"/>
-      <c r="D330" s="4" t="inlineStr"/>
-      <c r="E330" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F330" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C330" s="3" t="inlineStr"/>
+      <c r="D330" s="3" t="inlineStr"/>
+      <c r="E330" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F330" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="4" t="inlineStr">
+      <c r="A331" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B331" s="4" t="n">
+      <c r="B331" s="3" t="n">
         <v>11579255</v>
       </c>
-      <c r="C331" s="4" t="inlineStr"/>
-      <c r="D331" s="4" t="inlineStr"/>
-      <c r="E331" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F331" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C331" s="3" t="inlineStr"/>
+      <c r="D331" s="3" t="inlineStr"/>
+      <c r="E331" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F331" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -8251,24 +8347,24 @@
       </c>
     </row>
     <row r="342">
-      <c r="A342" s="4" t="inlineStr">
+      <c r="A342" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B342" s="4" t="n">
+      <c r="B342" s="3" t="n">
         <v>7018146</v>
       </c>
-      <c r="C342" s="4" t="inlineStr"/>
-      <c r="D342" s="4" t="inlineStr"/>
-      <c r="E342" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F342" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C342" s="3" t="inlineStr"/>
+      <c r="D342" s="3" t="inlineStr"/>
+      <c r="E342" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F342" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10085,464 +10181,488 @@
       </c>
     </row>
     <row r="425">
-      <c r="A425" s="4" t="inlineStr">
+      <c r="A425" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B425" s="4" t="n">
+      <c r="B425" s="3" t="n">
         <v>6947174</v>
       </c>
-      <c r="C425" s="4" t="inlineStr"/>
-      <c r="D425" s="4" t="inlineStr"/>
-      <c r="E425" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F425" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C425" s="3" t="inlineStr"/>
+      <c r="D425" s="3" t="inlineStr"/>
+      <c r="E425" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F425" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="426">
-      <c r="A426" s="4" t="inlineStr">
+      <c r="A426" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B426" s="4" t="n">
+      <c r="B426" s="3" t="n">
         <v>9349047</v>
       </c>
-      <c r="C426" s="4" t="inlineStr"/>
-      <c r="D426" s="4" t="inlineStr"/>
-      <c r="E426" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F426" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C426" s="3" t="inlineStr"/>
+      <c r="D426" s="3" t="inlineStr"/>
+      <c r="E426" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F426" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="427">
-      <c r="A427" s="4" t="inlineStr">
+      <c r="A427" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B427" s="4" t="n">
+      <c r="B427" s="2" t="n">
         <v>9349093</v>
       </c>
-      <c r="C427" s="4" t="inlineStr"/>
-      <c r="D427" s="4" t="inlineStr"/>
-      <c r="E427" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F427" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>316443916</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>Electrolux Range Relay Board - 316443916</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 9349093; fits EW30 range models per listing</t>
         </is>
       </c>
     </row>
     <row r="428">
-      <c r="A428" s="4" t="inlineStr">
+      <c r="A428" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B428" s="4" t="n">
+      <c r="B428" s="3" t="n">
         <v>6947945</v>
       </c>
-      <c r="C428" s="4" t="inlineStr"/>
-      <c r="D428" s="4" t="inlineStr"/>
-      <c r="E428" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F428" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C428" s="3" t="inlineStr"/>
+      <c r="D428" s="3" t="inlineStr"/>
+      <c r="E428" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F428" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="429">
-      <c r="A429" s="4" t="inlineStr">
+      <c r="A429" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B429" s="4" t="n">
+      <c r="B429" s="3" t="n">
         <v>8089749</v>
       </c>
-      <c r="C429" s="4" t="inlineStr"/>
-      <c r="D429" s="4" t="inlineStr"/>
-      <c r="E429" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F429" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C429" s="3" t="inlineStr"/>
+      <c r="D429" s="3" t="inlineStr"/>
+      <c r="E429" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F429" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="430">
-      <c r="A430" s="4" t="inlineStr">
+      <c r="A430" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B430" s="4" t="n">
+      <c r="B430" s="3" t="n">
         <v>9349296</v>
       </c>
-      <c r="C430" s="4" t="inlineStr"/>
-      <c r="D430" s="4" t="inlineStr"/>
-      <c r="E430" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F430" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C430" s="3" t="inlineStr"/>
+      <c r="D430" s="3" t="inlineStr"/>
+      <c r="E430" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F430" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="431">
-      <c r="A431" s="4" t="inlineStr">
+      <c r="A431" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B431" s="4" t="n">
+      <c r="B431" s="3" t="n">
         <v>11654521</v>
       </c>
-      <c r="C431" s="4" t="inlineStr"/>
-      <c r="D431" s="4" t="inlineStr"/>
-      <c r="E431" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F431" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C431" s="3" t="inlineStr"/>
+      <c r="D431" s="3" t="inlineStr"/>
+      <c r="E431" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F431" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="432">
-      <c r="A432" s="4" t="inlineStr">
+      <c r="A432" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B432" s="4" t="n">
+      <c r="B432" s="3" t="n">
         <v>9349191</v>
       </c>
-      <c r="C432" s="4" t="inlineStr"/>
-      <c r="D432" s="4" t="inlineStr"/>
-      <c r="E432" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F432" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C432" s="3" t="inlineStr"/>
+      <c r="D432" s="3" t="inlineStr"/>
+      <c r="E432" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F432" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="433">
-      <c r="A433" s="4" t="inlineStr">
+      <c r="A433" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B433" s="4" t="n">
+      <c r="B433" s="3" t="n">
         <v>9349282</v>
       </c>
-      <c r="C433" s="4" t="inlineStr"/>
-      <c r="D433" s="4" t="inlineStr"/>
-      <c r="E433" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F433" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C433" s="3" t="inlineStr"/>
+      <c r="D433" s="3" t="inlineStr"/>
+      <c r="E433" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F433" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="434">
-      <c r="A434" s="4" t="inlineStr">
+      <c r="A434" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B434" s="4" t="n">
+      <c r="B434" s="3" t="n">
         <v>9349290</v>
       </c>
-      <c r="C434" s="4" t="inlineStr"/>
-      <c r="D434" s="4" t="inlineStr"/>
-      <c r="E434" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F434" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C434" s="3" t="inlineStr"/>
+      <c r="D434" s="3" t="inlineStr"/>
+      <c r="E434" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F434" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="435">
-      <c r="A435" s="4" t="inlineStr">
+      <c r="A435" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B435" s="4" t="n">
+      <c r="B435" s="3" t="n">
         <v>9349682</v>
       </c>
-      <c r="C435" s="4" t="inlineStr"/>
-      <c r="D435" s="4" t="inlineStr"/>
-      <c r="E435" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F435" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C435" s="3" t="inlineStr"/>
+      <c r="D435" s="3" t="inlineStr"/>
+      <c r="E435" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F435" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="436">
-      <c r="A436" s="4" t="inlineStr">
+      <c r="A436" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B436" s="4" t="n">
+      <c r="B436" s="2" t="n">
         <v>9350077</v>
       </c>
-      <c r="C436" s="4" t="inlineStr"/>
-      <c r="D436" s="4" t="inlineStr"/>
-      <c r="E436" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F436" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C436" s="2" t="inlineStr">
+        <is>
+          <t>316560118</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>Electrolux Range Electronic Controller (ES540) - 316560118</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 9350077 listed under brand Electrolux; fits FGGF-series ranges per listing</t>
         </is>
       </c>
     </row>
     <row r="437">
-      <c r="A437" s="4" t="inlineStr">
+      <c r="A437" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B437" s="4" t="n">
+      <c r="B437" s="3" t="n">
         <v>9835061</v>
       </c>
-      <c r="C437" s="4" t="inlineStr"/>
-      <c r="D437" s="4" t="inlineStr"/>
-      <c r="E437" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F437" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C437" s="3" t="inlineStr"/>
+      <c r="D437" s="3" t="inlineStr"/>
+      <c r="E437" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F437" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="438">
-      <c r="A438" s="4" t="inlineStr">
+      <c r="A438" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B438" s="4" t="n">
+      <c r="B438" s="2" t="n">
         <v>9350269</v>
       </c>
-      <c r="C438" s="4" t="inlineStr"/>
-      <c r="D438" s="4" t="inlineStr"/>
-      <c r="E438" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F438" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C438" s="2" t="inlineStr">
+        <is>
+          <t>316576610</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>Electrolux Range Electronic Controller (ES630) - 316576610</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 9350269 listed under brand Electrolux; fits EW30 range models per listing</t>
         </is>
       </c>
     </row>
     <row r="439">
-      <c r="A439" s="4" t="inlineStr">
+      <c r="A439" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B439" s="4" t="n">
+      <c r="B439" s="3" t="n">
         <v>9835036</v>
       </c>
-      <c r="C439" s="4" t="inlineStr"/>
-      <c r="D439" s="4" t="inlineStr"/>
-      <c r="E439" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F439" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C439" s="3" t="inlineStr"/>
+      <c r="D439" s="3" t="inlineStr"/>
+      <c r="E439" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F439" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="440">
-      <c r="A440" s="4" t="inlineStr">
+      <c r="A440" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B440" s="4" t="n">
+      <c r="B440" s="3" t="n">
         <v>9835062</v>
       </c>
-      <c r="C440" s="4" t="inlineStr"/>
-      <c r="D440" s="4" t="inlineStr"/>
-      <c r="E440" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F440" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C440" s="3" t="inlineStr"/>
+      <c r="D440" s="3" t="inlineStr"/>
+      <c r="E440" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F440" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="441">
-      <c r="A441" s="4" t="inlineStr">
+      <c r="A441" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B441" s="4" t="n">
+      <c r="B441" s="3" t="n">
         <v>9835005</v>
       </c>
-      <c r="C441" s="4" t="inlineStr"/>
-      <c r="D441" s="4" t="inlineStr"/>
-      <c r="E441" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F441" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C441" s="3" t="inlineStr"/>
+      <c r="D441" s="3" t="inlineStr"/>
+      <c r="E441" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F441" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="442">
-      <c r="A442" s="4" t="inlineStr">
+      <c r="A442" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B442" s="4" t="n">
+      <c r="B442" s="3" t="n">
         <v>9835004</v>
       </c>
-      <c r="C442" s="4" t="inlineStr"/>
-      <c r="D442" s="4" t="inlineStr"/>
-      <c r="E442" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F442" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C442" s="3" t="inlineStr"/>
+      <c r="D442" s="3" t="inlineStr"/>
+      <c r="E442" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F442" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="443">
-      <c r="A443" s="4" t="inlineStr">
+      <c r="A443" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B443" s="4" t="n">
+      <c r="B443" s="3" t="n">
         <v>9350706</v>
       </c>
-      <c r="C443" s="4" t="inlineStr"/>
-      <c r="D443" s="4" t="inlineStr"/>
-      <c r="E443" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F443" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C443" s="3" t="inlineStr"/>
+      <c r="D443" s="3" t="inlineStr"/>
+      <c r="E443" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F443" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="444">
-      <c r="A444" s="4" t="inlineStr">
+      <c r="A444" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B444" s="4" t="n">
+      <c r="B444" s="3" t="n">
         <v>6948923</v>
       </c>
-      <c r="C444" s="4" t="inlineStr"/>
-      <c r="D444" s="4" t="inlineStr"/>
-      <c r="E444" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F444" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C444" s="3" t="inlineStr"/>
+      <c r="D444" s="3" t="inlineStr"/>
+      <c r="E444" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F444" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="445">
-      <c r="A445" s="4" t="inlineStr">
+      <c r="A445" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B445" s="4" t="n">
+      <c r="B445" s="3" t="n">
         <v>6953830</v>
       </c>
-      <c r="C445" s="4" t="inlineStr"/>
-      <c r="D445" s="4" t="inlineStr"/>
-      <c r="E445" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F445" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C445" s="3" t="inlineStr"/>
+      <c r="D445" s="3" t="inlineStr"/>
+      <c r="E445" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F445" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10569,24 +10689,32 @@
       </c>
     </row>
     <row r="447">
-      <c r="A447" s="4" t="inlineStr">
+      <c r="A447" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B447" s="4" t="n">
+      <c r="B447" s="3" t="n">
         <v>10168877</v>
       </c>
-      <c r="C447" s="4" t="inlineStr"/>
-      <c r="D447" s="4" t="inlineStr"/>
-      <c r="E447" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F447" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C447" s="3" t="inlineStr">
+        <is>
+          <t>5304495520</t>
+        </is>
+      </c>
+      <c r="D447" s="3" t="inlineStr">
+        <is>
+          <t>Electrolux Range Clock Kit (ES540) - 5304495520</t>
+        </is>
+      </c>
+      <c r="E447" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F447" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 10168877; listing names ES540 (range control) but no appliance type stated - verify</t>
         </is>
       </c>
     </row>
@@ -10613,24 +10741,24 @@
       </c>
     </row>
     <row r="449">
-      <c r="A449" s="4" t="inlineStr">
+      <c r="A449" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B449" s="4" t="n">
+      <c r="B449" s="3" t="n">
         <v>10878840</v>
       </c>
-      <c r="C449" s="4" t="inlineStr"/>
-      <c r="D449" s="4" t="inlineStr"/>
-      <c r="E449" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F449" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C449" s="3" t="inlineStr"/>
+      <c r="D449" s="3" t="inlineStr"/>
+      <c r="E449" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F449" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10657,178 +10785,194 @@
       </c>
     </row>
     <row r="451">
-      <c r="A451" s="4" t="inlineStr">
+      <c r="A451" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B451" s="4" t="n">
+      <c r="B451" s="3" t="n">
         <v>11578315</v>
       </c>
-      <c r="C451" s="4" t="inlineStr"/>
-      <c r="D451" s="4" t="inlineStr"/>
-      <c r="E451" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F451" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C451" s="3" t="inlineStr"/>
+      <c r="D451" s="3" t="inlineStr"/>
+      <c r="E451" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F451" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="452">
-      <c r="A452" s="4" t="inlineStr">
+      <c r="A452" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B452" s="4" t="n">
+      <c r="B452" s="2" t="n">
         <v>11578327</v>
       </c>
-      <c r="C452" s="4" t="inlineStr"/>
-      <c r="D452" s="4" t="inlineStr"/>
-      <c r="E452" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F452" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C452" s="2" t="inlineStr">
+        <is>
+          <t>5304511258</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>Electrolux Range SmoothTop Glass Assembly (Black) - 5304511258</t>
+        </is>
+      </c>
+      <c r="E452" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 11578327 listed under brand Electrolux</t>
         </is>
       </c>
     </row>
     <row r="453">
-      <c r="A453" s="4" t="inlineStr">
+      <c r="A453" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B453" s="4" t="n">
+      <c r="B453" s="3" t="n">
         <v>11578959</v>
       </c>
-      <c r="C453" s="4" t="inlineStr"/>
-      <c r="D453" s="4" t="inlineStr"/>
-      <c r="E453" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F453" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C453" s="3" t="inlineStr"/>
+      <c r="D453" s="3" t="inlineStr"/>
+      <c r="E453" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F453" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="454">
-      <c r="A454" s="4" t="inlineStr">
+      <c r="A454" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B454" s="4" t="n">
+      <c r="B454" s="3" t="n">
         <v>11579003</v>
       </c>
-      <c r="C454" s="4" t="inlineStr"/>
-      <c r="D454" s="4" t="inlineStr"/>
-      <c r="E454" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F454" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C454" s="3" t="inlineStr"/>
+      <c r="D454" s="3" t="inlineStr"/>
+      <c r="E454" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F454" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="455">
-      <c r="A455" s="4" t="inlineStr">
+      <c r="A455" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B455" s="4" t="n">
+      <c r="B455" s="3" t="n">
         <v>11654923</v>
       </c>
-      <c r="C455" s="4" t="inlineStr"/>
-      <c r="D455" s="4" t="inlineStr"/>
-      <c r="E455" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F455" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C455" s="3" t="inlineStr"/>
+      <c r="D455" s="3" t="inlineStr"/>
+      <c r="E455" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F455" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="456">
-      <c r="A456" s="4" t="inlineStr">
+      <c r="A456" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B456" s="4" t="n">
+      <c r="B456" s="3" t="n">
         <v>12444423</v>
       </c>
-      <c r="C456" s="4" t="inlineStr"/>
-      <c r="D456" s="4" t="inlineStr"/>
-      <c r="E456" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F456" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C456" s="3" t="inlineStr"/>
+      <c r="D456" s="3" t="inlineStr"/>
+      <c r="E456" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F456" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="457">
-      <c r="A457" s="4" t="inlineStr">
+      <c r="A457" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B457" s="4" t="n">
+      <c r="B457" s="3" t="n">
         <v>12619548</v>
       </c>
-      <c r="C457" s="4" t="inlineStr"/>
-      <c r="D457" s="4" t="inlineStr"/>
-      <c r="E457" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F457" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C457" s="3" t="inlineStr"/>
+      <c r="D457" s="3" t="inlineStr"/>
+      <c r="E457" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F457" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="458">
-      <c r="A458" s="4" t="inlineStr">
+      <c r="A458" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B458" s="4" t="n">
+      <c r="B458" s="3" t="n">
         <v>10879182</v>
       </c>
-      <c r="C458" s="4" t="inlineStr"/>
-      <c r="D458" s="4" t="inlineStr"/>
-      <c r="E458" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F458" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C458" s="3" t="inlineStr">
+        <is>
+          <t>807038640</t>
+        </is>
+      </c>
+      <c r="D458" s="3" t="inlineStr">
+        <is>
+          <t>Electrolux Cooktop SmoothTop Glass &amp; Steel Assembly - 807038640</t>
+        </is>
+      </c>
+      <c r="E458" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F458" s="3" t="inlineStr">
+        <is>
+          <t>Listing shows 10879182 as base part for model 807038640; single seller page</t>
         </is>
       </c>
     </row>
@@ -10877,46 +11021,46 @@
       </c>
     </row>
     <row r="461">
-      <c r="A461" s="4" t="inlineStr">
+      <c r="A461" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B461" s="4" t="n">
+      <c r="B461" s="3" t="n">
         <v>12896729</v>
       </c>
-      <c r="C461" s="4" t="inlineStr"/>
-      <c r="D461" s="4" t="inlineStr"/>
-      <c r="E461" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F461" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C461" s="3" t="inlineStr"/>
+      <c r="D461" s="3" t="inlineStr"/>
+      <c r="E461" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F461" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="462">
-      <c r="A462" s="4" t="inlineStr">
+      <c r="A462" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B462" s="4" t="n">
+      <c r="B462" s="3" t="n">
         <v>12431317</v>
       </c>
-      <c r="C462" s="4" t="inlineStr"/>
-      <c r="D462" s="4" t="inlineStr"/>
-      <c r="E462" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F462" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C462" s="3" t="inlineStr"/>
+      <c r="D462" s="3" t="inlineStr"/>
+      <c r="E462" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F462" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -10943,134 +11087,134 @@
       </c>
     </row>
     <row r="464">
-      <c r="A464" s="4" t="inlineStr">
+      <c r="A464" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B464" s="4" t="n">
+      <c r="B464" s="3" t="n">
         <v>10847476</v>
       </c>
-      <c r="C464" s="4" t="inlineStr"/>
-      <c r="D464" s="4" t="inlineStr"/>
-      <c r="E464" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F464" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C464" s="3" t="inlineStr"/>
+      <c r="D464" s="3" t="inlineStr"/>
+      <c r="E464" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F464" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="465">
-      <c r="A465" s="4" t="inlineStr">
+      <c r="A465" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B465" s="4" t="n">
+      <c r="B465" s="3" t="n">
         <v>9835037</v>
       </c>
-      <c r="C465" s="4" t="inlineStr"/>
-      <c r="D465" s="4" t="inlineStr"/>
-      <c r="E465" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F465" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C465" s="3" t="inlineStr"/>
+      <c r="D465" s="3" t="inlineStr"/>
+      <c r="E465" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F465" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="466">
-      <c r="A466" s="4" t="inlineStr">
+      <c r="A466" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B466" s="4" t="n">
+      <c r="B466" s="3" t="n">
         <v>11579255</v>
       </c>
-      <c r="C466" s="4" t="inlineStr"/>
-      <c r="D466" s="4" t="inlineStr"/>
-      <c r="E466" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F466" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C466" s="3" t="inlineStr"/>
+      <c r="D466" s="3" t="inlineStr"/>
+      <c r="E466" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F466" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="467">
-      <c r="A467" s="4" t="inlineStr">
+      <c r="A467" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B467" s="4" t="n">
+      <c r="B467" s="3" t="n">
         <v>12444096</v>
       </c>
-      <c r="C467" s="4" t="inlineStr"/>
-      <c r="D467" s="4" t="inlineStr"/>
-      <c r="E467" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F467" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C467" s="3" t="inlineStr"/>
+      <c r="D467" s="3" t="inlineStr"/>
+      <c r="E467" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F467" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="468">
-      <c r="A468" s="4" t="inlineStr">
+      <c r="A468" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B468" s="4" t="n">
+      <c r="B468" s="3" t="n">
         <v>12524352</v>
       </c>
-      <c r="C468" s="4" t="inlineStr"/>
-      <c r="D468" s="4" t="inlineStr"/>
-      <c r="E468" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F468" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C468" s="3" t="inlineStr"/>
+      <c r="D468" s="3" t="inlineStr"/>
+      <c r="E468" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F468" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="469">
-      <c r="A469" s="4" t="inlineStr">
+      <c r="A469" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B469" s="4" t="n">
+      <c r="B469" s="3" t="n">
         <v>13053983</v>
       </c>
-      <c r="C469" s="4" t="inlineStr"/>
-      <c r="D469" s="4" t="inlineStr"/>
-      <c r="E469" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F469" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C469" s="3" t="inlineStr"/>
+      <c r="D469" s="3" t="inlineStr"/>
+      <c r="E469" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F469" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Range collection H1 tags: Bosch lookups
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -6327,68 +6327,76 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="4" t="inlineStr">
+      <c r="A248" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B248" s="4" t="n">
+      <c r="B248" s="2" t="n">
         <v>12499480</v>
       </c>
-      <c r="C248" s="4" t="inlineStr"/>
-      <c r="D248" s="4" t="inlineStr"/>
-      <c r="E248" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F248" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>11033919</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>Bosch Oven Operating Module - 11033919</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 12499480; fits HBE5452UC series (built-in oven) per listing</t>
         </is>
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="4" t="inlineStr">
+      <c r="A249" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B249" s="4" t="n">
+      <c r="B249" s="3" t="n">
         <v>11597884</v>
       </c>
-      <c r="C249" s="4" t="inlineStr"/>
-      <c r="D249" s="4" t="inlineStr"/>
-      <c r="E249" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F249" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C249" s="3" t="inlineStr"/>
+      <c r="D249" s="3" t="inlineStr"/>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="4" t="inlineStr">
+      <c r="A250" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B250" s="4" t="n">
+      <c r="B250" s="3" t="n">
         <v>12469969</v>
       </c>
-      <c r="C250" s="4" t="inlineStr"/>
-      <c r="D250" s="4" t="inlineStr"/>
-      <c r="E250" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F250" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C250" s="3" t="inlineStr"/>
+      <c r="D250" s="3" t="inlineStr"/>
+      <c r="E250" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F250" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6481,24 +6489,24 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="4" t="inlineStr">
+      <c r="A255" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B255" s="4" t="n">
+      <c r="B255" s="3" t="n">
         <v>10130655</v>
       </c>
-      <c r="C255" s="4" t="inlineStr"/>
-      <c r="D255" s="4" t="inlineStr"/>
-      <c r="E255" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F255" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C255" s="3" t="inlineStr"/>
+      <c r="D255" s="3" t="inlineStr"/>
+      <c r="E255" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F255" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6695,90 +6703,98 @@
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="4" t="inlineStr">
+      <c r="A264" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B264" s="4" t="n">
+      <c r="B264" s="3" t="n">
         <v>11053935</v>
       </c>
-      <c r="C264" s="4" t="inlineStr"/>
-      <c r="D264" s="4" t="inlineStr"/>
-      <c r="E264" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F264" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C264" s="3" t="inlineStr"/>
+      <c r="D264" s="3" t="inlineStr"/>
+      <c r="E264" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F264" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="4" t="inlineStr">
+      <c r="A265" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B265" s="4" t="n">
+      <c r="B265" s="3" t="n">
         <v>11114498</v>
       </c>
-      <c r="C265" s="4" t="inlineStr"/>
-      <c r="D265" s="4" t="inlineStr"/>
-      <c r="E265" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F265" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C265" s="3" t="inlineStr"/>
+      <c r="D265" s="3" t="inlineStr"/>
+      <c r="E265" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F265" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="4" t="inlineStr">
+      <c r="A266" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B266" s="4" t="n">
+      <c r="B266" s="3" t="n">
         <v>11525561</v>
       </c>
-      <c r="C266" s="4" t="inlineStr"/>
-      <c r="D266" s="4" t="inlineStr"/>
-      <c r="E266" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F266" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>00618624</t>
+        </is>
+      </c>
+      <c r="D266" s="3" t="inlineStr">
+        <is>
+          <t>Bosch Ignition - 00618624</t>
+        </is>
+      </c>
+      <c r="E266" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F266" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 11525561; Encompass description truncated ("Ignition D") and appliance type not stated - verify</t>
         </is>
       </c>
     </row>
     <row r="267">
-      <c r="A267" s="4" t="inlineStr">
+      <c r="A267" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B267" s="4" t="n">
+      <c r="B267" s="3" t="n">
         <v>11535419</v>
       </c>
-      <c r="C267" s="4" t="inlineStr"/>
-      <c r="D267" s="4" t="inlineStr"/>
-      <c r="E267" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F267" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C267" s="3" t="inlineStr"/>
+      <c r="D267" s="3" t="inlineStr"/>
+      <c r="E267" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F267" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6805,90 +6821,98 @@
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="4" t="inlineStr">
+      <c r="A269" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B269" s="4" t="n">
+      <c r="B269" s="3" t="n">
         <v>11593512</v>
       </c>
-      <c r="C269" s="4" t="inlineStr"/>
-      <c r="D269" s="4" t="inlineStr"/>
-      <c r="E269" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F269" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C269" s="3" t="inlineStr"/>
+      <c r="D269" s="3" t="inlineStr"/>
+      <c r="E269" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F269" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="4" t="inlineStr">
+      <c r="A270" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B270" s="4" t="n">
+      <c r="B270" s="2" t="n">
         <v>11596813</v>
       </c>
-      <c r="C270" s="4" t="inlineStr"/>
-      <c r="D270" s="4" t="inlineStr"/>
-      <c r="E270" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F270" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>11020741</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>Bosch Oven Programmed Control Module - 11020741</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 11596813; fits HBL8461UC/HBN8451UC oven models per listing</t>
         </is>
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="4" t="inlineStr">
+      <c r="A271" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B271" s="4" t="n">
+      <c r="B271" s="3" t="n">
         <v>11598251</v>
       </c>
-      <c r="C271" s="4" t="inlineStr"/>
-      <c r="D271" s="4" t="inlineStr"/>
-      <c r="E271" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F271" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C271" s="3" t="inlineStr"/>
+      <c r="D271" s="3" t="inlineStr"/>
+      <c r="E271" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F271" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="4" t="inlineStr">
+      <c r="A272" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B272" s="4" t="n">
+      <c r="B272" s="3" t="n">
         <v>11598730</v>
       </c>
-      <c r="C272" s="4" t="inlineStr"/>
-      <c r="D272" s="4" t="inlineStr"/>
-      <c r="E272" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F272" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C272" s="3" t="inlineStr"/>
+      <c r="D272" s="3" t="inlineStr"/>
+      <c r="E272" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F272" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6915,46 +6939,46 @@
       </c>
     </row>
     <row r="274">
-      <c r="A274" s="4" t="inlineStr">
+      <c r="A274" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B274" s="4" t="n">
+      <c r="B274" s="3" t="n">
         <v>11598735</v>
       </c>
-      <c r="C274" s="4" t="inlineStr"/>
-      <c r="D274" s="4" t="inlineStr"/>
-      <c r="E274" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F274" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C274" s="3" t="inlineStr"/>
+      <c r="D274" s="3" t="inlineStr"/>
+      <c r="E274" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F274" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="4" t="inlineStr">
+      <c r="A275" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B275" s="4" t="n">
+      <c r="B275" s="3" t="n">
         <v>11598514</v>
       </c>
-      <c r="C275" s="4" t="inlineStr"/>
-      <c r="D275" s="4" t="inlineStr"/>
-      <c r="E275" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F275" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C275" s="3" t="inlineStr"/>
+      <c r="D275" s="3" t="inlineStr"/>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F275" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -6981,24 +7005,24 @@
       </c>
     </row>
     <row r="277">
-      <c r="A277" s="4" t="inlineStr">
+      <c r="A277" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B277" s="4" t="n">
+      <c r="B277" s="3" t="n">
         <v>11742617</v>
       </c>
-      <c r="C277" s="4" t="inlineStr"/>
-      <c r="D277" s="4" t="inlineStr"/>
-      <c r="E277" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F277" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C277" s="3" t="inlineStr"/>
+      <c r="D277" s="3" t="inlineStr"/>
+      <c r="E277" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F277" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -7033,68 +7057,76 @@
       </c>
     </row>
     <row r="279">
-      <c r="A279" s="4" t="inlineStr">
+      <c r="A279" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B279" s="4" t="n">
+      <c r="B279" s="3" t="n">
         <v>12499289</v>
       </c>
-      <c r="C279" s="4" t="inlineStr"/>
-      <c r="D279" s="4" t="inlineStr"/>
-      <c r="E279" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F279" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>11032521</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>Bosch Programmed Control Module - 11032521</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F279" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 12499289; listing fits mixed PRG/PRD dishwasher and oven models - verify appliance type</t>
         </is>
       </c>
     </row>
     <row r="280">
-      <c r="A280" s="4" t="inlineStr">
+      <c r="A280" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B280" s="4" t="n">
+      <c r="B280" s="3" t="n">
         <v>12501545</v>
       </c>
-      <c r="C280" s="4" t="inlineStr"/>
-      <c r="D280" s="4" t="inlineStr"/>
-      <c r="E280" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F280" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C280" s="3" t="inlineStr"/>
+      <c r="D280" s="3" t="inlineStr"/>
+      <c r="E280" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F280" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="4" t="inlineStr">
+      <c r="A281" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B281" s="4" t="n">
+      <c r="B281" s="3" t="n">
         <v>12499976</v>
       </c>
-      <c r="C281" s="4" t="inlineStr"/>
-      <c r="D281" s="4" t="inlineStr"/>
-      <c r="E281" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F281" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C281" s="3" t="inlineStr"/>
+      <c r="D281" s="3" t="inlineStr"/>
+      <c r="E281" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F281" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -7151,68 +7183,76 @@
       </c>
     </row>
     <row r="284">
-      <c r="A284" s="4" t="inlineStr">
+      <c r="A284" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B284" s="4" t="n">
+      <c r="B284" s="3" t="n">
         <v>12924181</v>
       </c>
-      <c r="C284" s="4" t="inlineStr"/>
-      <c r="D284" s="4" t="inlineStr"/>
-      <c r="E284" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F284" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C284" s="3" t="inlineStr"/>
+      <c r="D284" s="3" t="inlineStr"/>
+      <c r="E284" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F284" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="4" t="inlineStr">
+      <c r="A285" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B285" s="4" t="n">
+      <c r="B285" s="3" t="n">
         <v>12924176</v>
       </c>
-      <c r="C285" s="4" t="inlineStr"/>
-      <c r="D285" s="4" t="inlineStr"/>
-      <c r="E285" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F285" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C285" s="3" t="inlineStr"/>
+      <c r="D285" s="3" t="inlineStr"/>
+      <c r="E285" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F285" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="286">
-      <c r="A286" s="4" t="inlineStr">
+      <c r="A286" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B286" s="4" t="n">
+      <c r="B286" s="2" t="n">
         <v>12924300</v>
       </c>
-      <c r="C286" s="4" t="inlineStr"/>
-      <c r="D286" s="4" t="inlineStr"/>
-      <c r="E286" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F286" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>12037243</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>Bosch Range Programmed Control Module - 12037243</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 12924300; fits HGI8056UC/HGI8046UC models per listing</t>
         </is>
       </c>
     </row>
@@ -8345,90 +8385,106 @@
       </c>
     </row>
     <row r="335">
-      <c r="A335" s="4" t="inlineStr">
+      <c r="A335" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B335" s="4" t="n">
+      <c r="B335" s="3" t="n">
         <v>12487471</v>
       </c>
-      <c r="C335" s="4" t="inlineStr"/>
-      <c r="D335" s="4" t="inlineStr"/>
-      <c r="E335" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F335" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C335" s="3" t="inlineStr">
+        <is>
+          <t>00669416</t>
+        </is>
+      </c>
+      <c r="D335" s="3" t="inlineStr">
+        <is>
+          <t>Bosch Fan Motor - 00669416</t>
+        </is>
+      </c>
+      <c r="E335" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F335" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 12487471; fits VTN/VTI models - appliance type not stated, verify</t>
         </is>
       </c>
     </row>
     <row r="336">
-      <c r="A336" s="4" t="inlineStr">
+      <c r="A336" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B336" s="4" t="n">
+      <c r="B336" s="3" t="n">
         <v>12924782</v>
       </c>
-      <c r="C336" s="4" t="inlineStr"/>
-      <c r="D336" s="4" t="inlineStr"/>
-      <c r="E336" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F336" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C336" s="3" t="inlineStr"/>
+      <c r="D336" s="3" t="inlineStr"/>
+      <c r="E336" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F336" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="337">
-      <c r="A337" s="4" t="inlineStr">
+      <c r="A337" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B337" s="4" t="n">
+      <c r="B337" s="3" t="n">
         <v>12492721</v>
       </c>
-      <c r="C337" s="4" t="inlineStr"/>
-      <c r="D337" s="4" t="inlineStr"/>
-      <c r="E337" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F337" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C337" s="3" t="inlineStr"/>
+      <c r="D337" s="3" t="inlineStr"/>
+      <c r="E337" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F337" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="338">
-      <c r="A338" s="4" t="inlineStr">
+      <c r="A338" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B338" s="4" t="n">
+      <c r="B338" s="2" t="n">
         <v>12503030</v>
       </c>
-      <c r="C338" s="4" t="inlineStr"/>
-      <c r="D338" s="4" t="inlineStr"/>
-      <c r="E338" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F338" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>20000554</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>Bosch Oven Panel-Facia - 20000554</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 12503030; fits HBL-series oven models per listing</t>
         </is>
       </c>
     </row>
@@ -8529,90 +8585,90 @@
       </c>
     </row>
     <row r="343">
-      <c r="A343" s="4" t="inlineStr">
+      <c r="A343" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B343" s="4" t="n">
+      <c r="B343" s="3" t="n">
         <v>11437542</v>
       </c>
-      <c r="C343" s="4" t="inlineStr"/>
-      <c r="D343" s="4" t="inlineStr"/>
-      <c r="E343" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F343" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C343" s="3" t="inlineStr"/>
+      <c r="D343" s="3" t="inlineStr"/>
+      <c r="E343" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F343" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="344">
-      <c r="A344" s="4" t="inlineStr">
+      <c r="A344" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B344" s="4" t="n">
+      <c r="B344" s="3" t="n">
         <v>13372326</v>
       </c>
-      <c r="C344" s="4" t="inlineStr"/>
-      <c r="D344" s="4" t="inlineStr"/>
-      <c r="E344" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F344" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C344" s="3" t="inlineStr"/>
+      <c r="D344" s="3" t="inlineStr"/>
+      <c r="E344" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F344" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="345">
-      <c r="A345" s="4" t="inlineStr">
+      <c r="A345" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B345" s="4" t="n">
+      <c r="B345" s="3" t="n">
         <v>12923012</v>
       </c>
-      <c r="C345" s="4" t="inlineStr"/>
-      <c r="D345" s="4" t="inlineStr"/>
-      <c r="E345" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F345" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C345" s="3" t="inlineStr"/>
+      <c r="D345" s="3" t="inlineStr"/>
+      <c r="E345" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F345" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="346">
-      <c r="A346" s="4" t="inlineStr">
+      <c r="A346" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B346" s="4" t="n">
+      <c r="B346" s="3" t="n">
         <v>12923009</v>
       </c>
-      <c r="C346" s="4" t="inlineStr"/>
-      <c r="D346" s="4" t="inlineStr"/>
-      <c r="E346" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F346" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C346" s="3" t="inlineStr"/>
+      <c r="D346" s="3" t="inlineStr"/>
+      <c r="E346" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F346" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -8639,156 +8695,156 @@
       </c>
     </row>
     <row r="348">
-      <c r="A348" s="4" t="inlineStr">
+      <c r="A348" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B348" s="4" t="n">
+      <c r="B348" s="3" t="n">
         <v>14899112</v>
       </c>
-      <c r="C348" s="4" t="inlineStr"/>
-      <c r="D348" s="4" t="inlineStr"/>
-      <c r="E348" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F348" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C348" s="3" t="inlineStr"/>
+      <c r="D348" s="3" t="inlineStr"/>
+      <c r="E348" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F348" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="349">
-      <c r="A349" s="4" t="inlineStr">
+      <c r="A349" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B349" s="4" t="n">
+      <c r="B349" s="3" t="n">
         <v>13609473</v>
       </c>
-      <c r="C349" s="4" t="inlineStr"/>
-      <c r="D349" s="4" t="inlineStr"/>
-      <c r="E349" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F349" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C349" s="3" t="inlineStr"/>
+      <c r="D349" s="3" t="inlineStr"/>
+      <c r="E349" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F349" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="350">
-      <c r="A350" s="4" t="inlineStr">
+      <c r="A350" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B350" s="4" t="n">
+      <c r="B350" s="3" t="n">
         <v>12323195</v>
       </c>
-      <c r="C350" s="4" t="inlineStr"/>
-      <c r="D350" s="4" t="inlineStr"/>
-      <c r="E350" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F350" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C350" s="3" t="inlineStr"/>
+      <c r="D350" s="3" t="inlineStr"/>
+      <c r="E350" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F350" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="351">
-      <c r="A351" s="4" t="inlineStr">
+      <c r="A351" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B351" s="4" t="n">
+      <c r="B351" s="3" t="n">
         <v>12488482</v>
       </c>
-      <c r="C351" s="4" t="inlineStr"/>
-      <c r="D351" s="4" t="inlineStr"/>
-      <c r="E351" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F351" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C351" s="3" t="inlineStr"/>
+      <c r="D351" s="3" t="inlineStr"/>
+      <c r="E351" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F351" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="352">
-      <c r="A352" s="4" t="inlineStr">
+      <c r="A352" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B352" s="4" t="n">
+      <c r="B352" s="3" t="n">
         <v>12490537</v>
       </c>
-      <c r="C352" s="4" t="inlineStr"/>
-      <c r="D352" s="4" t="inlineStr"/>
-      <c r="E352" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F352" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C352" s="3" t="inlineStr"/>
+      <c r="D352" s="3" t="inlineStr"/>
+      <c r="E352" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F352" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="353">
-      <c r="A353" s="4" t="inlineStr">
+      <c r="A353" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B353" s="4" t="n">
+      <c r="B353" s="3" t="n">
         <v>12491052</v>
       </c>
-      <c r="C353" s="4" t="inlineStr"/>
-      <c r="D353" s="4" t="inlineStr"/>
-      <c r="E353" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F353" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C353" s="3" t="inlineStr"/>
+      <c r="D353" s="3" t="inlineStr"/>
+      <c r="E353" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F353" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="354">
-      <c r="A354" s="4" t="inlineStr">
+      <c r="A354" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B354" s="4" t="n">
+      <c r="B354" s="3" t="n">
         <v>12493839</v>
       </c>
-      <c r="C354" s="4" t="inlineStr"/>
-      <c r="D354" s="4" t="inlineStr"/>
-      <c r="E354" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F354" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C354" s="3" t="inlineStr"/>
+      <c r="D354" s="3" t="inlineStr"/>
+      <c r="E354" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F354" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Range collection H1 tags: finish remaining lookups
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,11 +46,6 @@
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -64,12 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5971,24 +5965,32 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="4" t="inlineStr">
+      <c r="A232" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B232" s="4" t="n">
+      <c r="B232" s="3" t="n">
         <v>11584932</v>
       </c>
-      <c r="C232" s="4" t="inlineStr"/>
-      <c r="D232" s="4" t="inlineStr"/>
-      <c r="E232" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F232" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>200559</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Piano Lav.S7H D1 Inox - 200559</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 11584932; description is Bertazzoni catalog wording, appliance type not stated - verify</t>
         </is>
       </c>
     </row>
@@ -6037,24 +6039,32 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="4" t="inlineStr">
+      <c r="A235" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B235" s="4" t="n">
+      <c r="B235" s="3" t="n">
         <v>12710552</v>
       </c>
-      <c r="C235" s="4" t="inlineStr"/>
-      <c r="D235" s="4" t="inlineStr"/>
-      <c r="E235" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F235" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>211256</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Work Table - 211256</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 12710552; appliance type not stated - verify</t>
         </is>
       </c>
     </row>
@@ -6081,24 +6091,24 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="4" t="inlineStr">
+      <c r="A237" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B237" s="4" t="n">
+      <c r="B237" s="3" t="n">
         <v>12320894</v>
       </c>
-      <c r="C237" s="4" t="inlineStr"/>
-      <c r="D237" s="4" t="inlineStr"/>
-      <c r="E237" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F237" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C237" s="3" t="inlineStr"/>
+      <c r="D237" s="3" t="inlineStr"/>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -8171,24 +8181,24 @@
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="4" t="inlineStr">
+      <c r="A326" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B326" s="4" t="n">
+      <c r="B326" s="3" t="n">
         <v>11830416</v>
       </c>
-      <c r="C326" s="4" t="inlineStr"/>
-      <c r="D326" s="4" t="inlineStr"/>
-      <c r="E326" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F326" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C326" s="3" t="inlineStr"/>
+      <c r="D326" s="3" t="inlineStr"/>
+      <c r="E326" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F326" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -8319,68 +8329,84 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="4" t="inlineStr">
+      <c r="A332" s="2" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B332" s="4" t="n">
+      <c r="B332" s="2" t="n">
         <v>11830415</v>
       </c>
-      <c r="C332" s="4" t="inlineStr"/>
-      <c r="D332" s="4" t="inlineStr"/>
-      <c r="E332" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F332" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>4410300337</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>Blomberg Cooktop Ceran Frame Burner Plate Group (White) - 4410300337</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 11830415 (blomberg.encompass.com listing)</t>
         </is>
       </c>
     </row>
     <row r="333">
-      <c r="A333" s="4" t="inlineStr">
+      <c r="A333" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B333" s="4" t="n">
+      <c r="B333" s="3" t="n">
         <v>12598403</v>
       </c>
-      <c r="C333" s="4" t="inlineStr"/>
-      <c r="D333" s="4" t="inlineStr"/>
-      <c r="E333" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F333" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C333" s="3" t="inlineStr"/>
+      <c r="D333" s="3" t="inlineStr"/>
+      <c r="E333" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F333" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="334">
-      <c r="A334" s="4" t="inlineStr">
+      <c r="A334" s="2" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B334" s="4" t="n">
+      <c r="B334" s="2" t="n">
         <v>11830418</v>
       </c>
-      <c r="C334" s="4" t="inlineStr"/>
-      <c r="D334" s="4" t="inlineStr"/>
-      <c r="E334" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F334" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>4410600053</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>Blomberg Cooktop Ceran Hob Burner Plate (Inox) - 4410600053</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 11830418 (blomberg.encompass.com listing)</t>
         </is>
       </c>
     </row>
@@ -8489,24 +8515,24 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="4" t="inlineStr">
+      <c r="A339" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B339" s="4" t="n">
+      <c r="B339" s="3" t="n">
         <v>12934311</v>
       </c>
-      <c r="C339" s="4" t="inlineStr"/>
-      <c r="D339" s="4" t="inlineStr"/>
-      <c r="E339" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F339" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C339" s="3" t="inlineStr"/>
+      <c r="D339" s="3" t="inlineStr"/>
+      <c r="E339" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F339" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -8849,376 +8875,384 @@
       </c>
     </row>
     <row r="355">
-      <c r="A355" s="4" t="inlineStr">
+      <c r="A355" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B355" s="4" t="n">
+      <c r="B355" s="3" t="n">
         <v>12493851</v>
       </c>
-      <c r="C355" s="4" t="inlineStr"/>
-      <c r="D355" s="4" t="inlineStr"/>
-      <c r="E355" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F355" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C355" s="3" t="inlineStr"/>
+      <c r="D355" s="3" t="inlineStr"/>
+      <c r="E355" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F355" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="356">
-      <c r="A356" s="4" t="inlineStr">
+      <c r="A356" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B356" s="4" t="n">
+      <c r="B356" s="3" t="n">
         <v>12494273</v>
       </c>
-      <c r="C356" s="4" t="inlineStr"/>
-      <c r="D356" s="4" t="inlineStr"/>
-      <c r="E356" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F356" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C356" s="3" t="inlineStr"/>
+      <c r="D356" s="3" t="inlineStr"/>
+      <c r="E356" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F356" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="357">
-      <c r="A357" s="4" t="inlineStr">
+      <c r="A357" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B357" s="4" t="n">
+      <c r="B357" s="3" t="n">
         <v>12497106</v>
       </c>
-      <c r="C357" s="4" t="inlineStr"/>
-      <c r="D357" s="4" t="inlineStr"/>
-      <c r="E357" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F357" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C357" s="3" t="inlineStr"/>
+      <c r="D357" s="3" t="inlineStr"/>
+      <c r="E357" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F357" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="358">
-      <c r="A358" s="4" t="inlineStr">
+      <c r="A358" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B358" s="4" t="n">
+      <c r="B358" s="3" t="n">
         <v>12502886</v>
       </c>
-      <c r="C358" s="4" t="inlineStr"/>
-      <c r="D358" s="4" t="inlineStr"/>
-      <c r="E358" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F358" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C358" s="3" t="inlineStr"/>
+      <c r="D358" s="3" t="inlineStr"/>
+      <c r="E358" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F358" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="359">
-      <c r="A359" s="4" t="inlineStr">
+      <c r="A359" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B359" s="4" t="n">
+      <c r="B359" s="2" t="n">
         <v>12503043</v>
       </c>
-      <c r="C359" s="4" t="inlineStr"/>
-      <c r="D359" s="4" t="inlineStr"/>
-      <c r="E359" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F359" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>20000598</t>
+        </is>
+      </c>
+      <c r="D359" s="2" t="inlineStr">
+        <is>
+          <t>Bosch Oven Front Panel - 20000598</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F359" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 12503043; fits HEI8056U oven models per listing</t>
         </is>
       </c>
     </row>
     <row r="360">
-      <c r="A360" s="4" t="inlineStr">
+      <c r="A360" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B360" s="4" t="n">
+      <c r="B360" s="3" t="n">
         <v>12503044</v>
       </c>
-      <c r="C360" s="4" t="inlineStr"/>
-      <c r="D360" s="4" t="inlineStr"/>
-      <c r="E360" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F360" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C360" s="3" t="inlineStr"/>
+      <c r="D360" s="3" t="inlineStr"/>
+      <c r="E360" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F360" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="361">
-      <c r="A361" s="4" t="inlineStr">
+      <c r="A361" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B361" s="4" t="n">
+      <c r="B361" s="3" t="n">
         <v>11525725</v>
       </c>
-      <c r="C361" s="4" t="inlineStr"/>
-      <c r="D361" s="4" t="inlineStr"/>
-      <c r="E361" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F361" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C361" s="3" t="inlineStr"/>
+      <c r="D361" s="3" t="inlineStr"/>
+      <c r="E361" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F361" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="362">
-      <c r="A362" s="4" t="inlineStr">
+      <c r="A362" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B362" s="4" t="n">
+      <c r="B362" s="3" t="n">
         <v>11598061</v>
       </c>
-      <c r="C362" s="4" t="inlineStr"/>
-      <c r="D362" s="4" t="inlineStr"/>
-      <c r="E362" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F362" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C362" s="3" t="inlineStr"/>
+      <c r="D362" s="3" t="inlineStr"/>
+      <c r="E362" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F362" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="363">
-      <c r="A363" s="4" t="inlineStr">
+      <c r="A363" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B363" s="4" t="n">
+      <c r="B363" s="3" t="n">
         <v>14894572</v>
       </c>
-      <c r="C363" s="4" t="inlineStr"/>
-      <c r="D363" s="4" t="inlineStr"/>
-      <c r="E363" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F363" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C363" s="3" t="inlineStr"/>
+      <c r="D363" s="3" t="inlineStr"/>
+      <c r="E363" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F363" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="364">
-      <c r="A364" s="4" t="inlineStr">
+      <c r="A364" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B364" s="4" t="n">
+      <c r="B364" s="3" t="n">
         <v>14894506</v>
       </c>
-      <c r="C364" s="4" t="inlineStr"/>
-      <c r="D364" s="4" t="inlineStr"/>
-      <c r="E364" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F364" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C364" s="3" t="inlineStr"/>
+      <c r="D364" s="3" t="inlineStr"/>
+      <c r="E364" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F364" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="365">
-      <c r="A365" s="4" t="inlineStr">
+      <c r="A365" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B365" s="4" t="n">
+      <c r="B365" s="3" t="n">
         <v>14894576</v>
       </c>
-      <c r="C365" s="4" t="inlineStr"/>
-      <c r="D365" s="4" t="inlineStr"/>
-      <c r="E365" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F365" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C365" s="3" t="inlineStr"/>
+      <c r="D365" s="3" t="inlineStr"/>
+      <c r="E365" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F365" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="366">
-      <c r="A366" s="4" t="inlineStr">
+      <c r="A366" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B366" s="4" t="n">
+      <c r="B366" s="3" t="n">
         <v>14896732</v>
       </c>
-      <c r="C366" s="4" t="inlineStr"/>
-      <c r="D366" s="4" t="inlineStr"/>
-      <c r="E366" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F366" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C366" s="3" t="inlineStr"/>
+      <c r="D366" s="3" t="inlineStr"/>
+      <c r="E366" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F366" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="367">
-      <c r="A367" s="4" t="inlineStr">
+      <c r="A367" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B367" s="4" t="n">
+      <c r="B367" s="3" t="n">
         <v>13589307</v>
       </c>
-      <c r="C367" s="4" t="inlineStr"/>
-      <c r="D367" s="4" t="inlineStr"/>
-      <c r="E367" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F367" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C367" s="3" t="inlineStr"/>
+      <c r="D367" s="3" t="inlineStr"/>
+      <c r="E367" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F367" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="368">
-      <c r="A368" s="4" t="inlineStr">
+      <c r="A368" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B368" s="4" t="n">
+      <c r="B368" s="3" t="n">
         <v>12709492</v>
       </c>
-      <c r="C368" s="4" t="inlineStr"/>
-      <c r="D368" s="4" t="inlineStr"/>
-      <c r="E368" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F368" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C368" s="3" t="inlineStr"/>
+      <c r="D368" s="3" t="inlineStr"/>
+      <c r="E368" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F368" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="369">
-      <c r="A369" s="4" t="inlineStr">
+      <c r="A369" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B369" s="4" t="n">
+      <c r="B369" s="3" t="n">
         <v>12709498</v>
       </c>
-      <c r="C369" s="4" t="inlineStr"/>
-      <c r="D369" s="4" t="inlineStr"/>
-      <c r="E369" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F369" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C369" s="3" t="inlineStr"/>
+      <c r="D369" s="3" t="inlineStr"/>
+      <c r="E369" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F369" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="370">
-      <c r="A370" s="4" t="inlineStr">
+      <c r="A370" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B370" s="4" t="n">
+      <c r="B370" s="3" t="n">
         <v>12709509</v>
       </c>
-      <c r="C370" s="4" t="inlineStr"/>
-      <c r="D370" s="4" t="inlineStr"/>
-      <c r="E370" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F370" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C370" s="3" t="inlineStr"/>
+      <c r="D370" s="3" t="inlineStr"/>
+      <c r="E370" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F370" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="371">
-      <c r="A371" s="4" t="inlineStr">
+      <c r="A371" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B371" s="4" t="n">
+      <c r="B371" s="3" t="n">
         <v>13393136</v>
       </c>
-      <c r="C371" s="4" t="inlineStr"/>
-      <c r="D371" s="4" t="inlineStr"/>
-      <c r="E371" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F371" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C371" s="3" t="inlineStr"/>
+      <c r="D371" s="3" t="inlineStr"/>
+      <c r="E371" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F371" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
@@ -9245,1124 +9279,1196 @@
       </c>
     </row>
     <row r="373">
-      <c r="A373" s="4" t="inlineStr">
+      <c r="A373" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B373" s="4" t="n">
+      <c r="B373" s="3" t="n">
         <v>12934269</v>
       </c>
-      <c r="C373" s="4" t="inlineStr"/>
-      <c r="D373" s="4" t="inlineStr"/>
-      <c r="E373" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F373" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C373" s="3" t="inlineStr"/>
+      <c r="D373" s="3" t="inlineStr"/>
+      <c r="E373" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F373" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="374">
-      <c r="A374" s="4" t="inlineStr">
+      <c r="A374" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B374" s="4" t="n">
+      <c r="B374" s="3" t="n">
         <v>11584900</v>
       </c>
-      <c r="C374" s="4" t="inlineStr"/>
-      <c r="D374" s="4" t="inlineStr"/>
-      <c r="E374" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F374" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C374" s="3" t="inlineStr"/>
+      <c r="D374" s="3" t="inlineStr"/>
+      <c r="E374" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F374" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="375">
-      <c r="A375" s="4" t="inlineStr">
+      <c r="A375" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B375" s="4" t="n">
+      <c r="B375" s="3" t="n">
         <v>11584917</v>
       </c>
-      <c r="C375" s="4" t="inlineStr"/>
-      <c r="D375" s="4" t="inlineStr"/>
-      <c r="E375" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F375" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C375" s="3" t="inlineStr"/>
+      <c r="D375" s="3" t="inlineStr"/>
+      <c r="E375" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F375" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="376">
-      <c r="A376" s="4" t="inlineStr">
+      <c r="A376" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B376" s="4" t="n">
+      <c r="B376" s="3" t="n">
         <v>11584929</v>
       </c>
-      <c r="C376" s="4" t="inlineStr"/>
-      <c r="D376" s="4" t="inlineStr"/>
-      <c r="E376" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F376" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C376" s="3" t="inlineStr"/>
+      <c r="D376" s="3" t="inlineStr"/>
+      <c r="E376" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F376" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="377">
-      <c r="A377" s="4" t="inlineStr">
+      <c r="A377" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B377" s="4" t="n">
+      <c r="B377" s="3" t="n">
         <v>11584915</v>
       </c>
-      <c r="C377" s="4" t="inlineStr"/>
-      <c r="D377" s="4" t="inlineStr"/>
-      <c r="E377" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F377" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C377" s="3" t="inlineStr"/>
+      <c r="D377" s="3" t="inlineStr"/>
+      <c r="E377" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F377" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="378">
-      <c r="A378" s="4" t="inlineStr">
+      <c r="A378" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B378" s="4" t="n">
+      <c r="B378" s="3" t="n">
         <v>11584920</v>
       </c>
-      <c r="C378" s="4" t="inlineStr"/>
-      <c r="D378" s="4" t="inlineStr"/>
-      <c r="E378" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F378" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C378" s="3" t="inlineStr"/>
+      <c r="D378" s="3" t="inlineStr"/>
+      <c r="E378" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F378" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="379">
-      <c r="A379" s="4" t="inlineStr">
+      <c r="A379" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B379" s="4" t="n">
+      <c r="B379" s="3" t="n">
         <v>11584897</v>
       </c>
-      <c r="C379" s="4" t="inlineStr"/>
-      <c r="D379" s="4" t="inlineStr"/>
-      <c r="E379" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F379" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C379" s="3" t="inlineStr"/>
+      <c r="D379" s="3" t="inlineStr"/>
+      <c r="E379" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F379" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="380">
-      <c r="A380" s="4" t="inlineStr">
+      <c r="A380" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B380" s="4" t="n">
+      <c r="B380" s="2" t="n">
         <v>11584921</v>
       </c>
-      <c r="C380" s="4" t="inlineStr"/>
-      <c r="D380" s="4" t="inlineStr"/>
-      <c r="E380" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F380" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t>128027</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Porta Forno Std1 Dx Pro Arancione - 128027</t>
+        </is>
+      </c>
+      <c r="E380" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 11584921; oven door, fits PROF486 range models per listing</t>
         </is>
       </c>
     </row>
     <row r="381">
-      <c r="A381" s="4" t="inlineStr">
+      <c r="A381" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B381" s="4" t="n">
+      <c r="B381" s="3" t="n">
         <v>11584928</v>
       </c>
-      <c r="C381" s="4" t="inlineStr"/>
-      <c r="D381" s="4" t="inlineStr"/>
-      <c r="E381" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F381" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C381" s="3" t="inlineStr"/>
+      <c r="D381" s="3" t="inlineStr"/>
+      <c r="E381" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F381" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="382">
-      <c r="A382" s="4" t="inlineStr">
+      <c r="A382" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B382" s="4" t="n">
+      <c r="B382" s="3" t="n">
         <v>12320940</v>
       </c>
-      <c r="C382" s="4" t="inlineStr"/>
-      <c r="D382" s="4" t="inlineStr"/>
-      <c r="E382" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F382" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C382" s="3" t="inlineStr"/>
+      <c r="D382" s="3" t="inlineStr"/>
+      <c r="E382" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F382" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="383">
-      <c r="A383" s="4" t="inlineStr">
+      <c r="A383" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B383" s="4" t="n">
+      <c r="B383" s="3" t="n">
         <v>12320899</v>
       </c>
-      <c r="C383" s="4" t="inlineStr"/>
-      <c r="D383" s="4" t="inlineStr"/>
-      <c r="E383" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F383" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C383" s="3" t="inlineStr"/>
+      <c r="D383" s="3" t="inlineStr"/>
+      <c r="E383" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F383" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="384">
-      <c r="A384" s="4" t="inlineStr">
+      <c r="A384" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B384" s="4" t="n">
+      <c r="B384" s="3" t="n">
         <v>11584904</v>
       </c>
-      <c r="C384" s="4" t="inlineStr"/>
-      <c r="D384" s="4" t="inlineStr"/>
-      <c r="E384" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F384" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C384" s="3" t="inlineStr"/>
+      <c r="D384" s="3" t="inlineStr"/>
+      <c r="E384" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F384" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="385">
-      <c r="A385" s="4" t="inlineStr">
+      <c r="A385" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B385" s="4" t="n">
+      <c r="B385" s="3" t="n">
         <v>11584919</v>
       </c>
-      <c r="C385" s="4" t="inlineStr"/>
-      <c r="D385" s="4" t="inlineStr"/>
-      <c r="E385" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F385" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C385" s="3" t="inlineStr"/>
+      <c r="D385" s="3" t="inlineStr"/>
+      <c r="E385" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F385" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="386">
-      <c r="A386" s="4" t="inlineStr">
+      <c r="A386" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B386" s="4" t="n">
+      <c r="B386" s="2" t="n">
         <v>12319102</v>
       </c>
-      <c r="C386" s="4" t="inlineStr"/>
-      <c r="D386" s="4" t="inlineStr"/>
-      <c r="E386" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F386" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>128027-DA</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Outer Right Oven Door Assembly - 128027-DA</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 12319102; fits PROF486 range models per listing</t>
         </is>
       </c>
     </row>
     <row r="387">
-      <c r="A387" s="4" t="inlineStr">
+      <c r="A387" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B387" s="4" t="n">
+      <c r="B387" s="3" t="n">
         <v>12319103</v>
       </c>
-      <c r="C387" s="4" t="inlineStr"/>
-      <c r="D387" s="4" t="inlineStr"/>
-      <c r="E387" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F387" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C387" s="3" t="inlineStr"/>
+      <c r="D387" s="3" t="inlineStr"/>
+      <c r="E387" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F387" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="388">
-      <c r="A388" s="4" t="inlineStr">
+      <c r="A388" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B388" s="4" t="n">
+      <c r="B388" s="3" t="n">
         <v>12319088</v>
       </c>
-      <c r="C388" s="4" t="inlineStr"/>
-      <c r="D388" s="4" t="inlineStr"/>
-      <c r="E388" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F388" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C388" s="3" t="inlineStr"/>
+      <c r="D388" s="3" t="inlineStr"/>
+      <c r="E388" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F388" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="389">
-      <c r="A389" s="4" t="inlineStr">
+      <c r="A389" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B389" s="4" t="n">
+      <c r="B389" s="3" t="n">
         <v>12319100</v>
       </c>
-      <c r="C389" s="4" t="inlineStr"/>
-      <c r="D389" s="4" t="inlineStr"/>
-      <c r="E389" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F389" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C389" s="3" t="inlineStr">
+        <is>
+          <t>128021-DA</t>
+        </is>
+      </c>
+      <c r="D389" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Outer Right Oven Door Assembly - 128021-DA</t>
+        </is>
+      </c>
+      <c r="E389" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F389" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 12319100; fitment models not shown - appliance type assumed from oven door family, verify</t>
         </is>
       </c>
     </row>
     <row r="390">
-      <c r="A390" s="4" t="inlineStr">
+      <c r="A390" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B390" s="4" t="n">
+      <c r="B390" s="3" t="n">
         <v>12320897</v>
       </c>
-      <c r="C390" s="4" t="inlineStr"/>
-      <c r="D390" s="4" t="inlineStr"/>
-      <c r="E390" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F390" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C390" s="3" t="inlineStr"/>
+      <c r="D390" s="3" t="inlineStr"/>
+      <c r="E390" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F390" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="391">
-      <c r="A391" s="4" t="inlineStr">
+      <c r="A391" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B391" s="4" t="n">
+      <c r="B391" s="3" t="n">
         <v>12319095</v>
       </c>
-      <c r="C391" s="4" t="inlineStr"/>
-      <c r="D391" s="4" t="inlineStr"/>
-      <c r="E391" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F391" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C391" s="3" t="inlineStr"/>
+      <c r="D391" s="3" t="inlineStr"/>
+      <c r="E391" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F391" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="392">
-      <c r="A392" s="4" t="inlineStr">
+      <c r="A392" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B392" s="4" t="n">
+      <c r="B392" s="3" t="n">
         <v>12319101</v>
       </c>
-      <c r="C392" s="4" t="inlineStr"/>
-      <c r="D392" s="4" t="inlineStr"/>
-      <c r="E392" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F392" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C392" s="3" t="inlineStr"/>
+      <c r="D392" s="3" t="inlineStr"/>
+      <c r="E392" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F392" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="393">
-      <c r="A393" s="4" t="inlineStr">
+      <c r="A393" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B393" s="4" t="n">
+      <c r="B393" s="3" t="n">
         <v>12607236</v>
       </c>
-      <c r="C393" s="4" t="inlineStr"/>
-      <c r="D393" s="4" t="inlineStr"/>
-      <c r="E393" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F393" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C393" s="3" t="inlineStr"/>
+      <c r="D393" s="3" t="inlineStr"/>
+      <c r="E393" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F393" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="394">
-      <c r="A394" s="4" t="inlineStr">
+      <c r="A394" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B394" s="4" t="n">
+      <c r="B394" s="3" t="n">
         <v>12524602</v>
       </c>
-      <c r="C394" s="4" t="inlineStr"/>
-      <c r="D394" s="4" t="inlineStr"/>
-      <c r="E394" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F394" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C394" s="3" t="inlineStr"/>
+      <c r="D394" s="3" t="inlineStr"/>
+      <c r="E394" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F394" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="395">
-      <c r="A395" s="4" t="inlineStr">
+      <c r="A395" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B395" s="4" t="n">
+      <c r="B395" s="3" t="n">
         <v>11525845</v>
       </c>
-      <c r="C395" s="4" t="inlineStr"/>
-      <c r="D395" s="4" t="inlineStr"/>
-      <c r="E395" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F395" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C395" s="3" t="inlineStr">
+        <is>
+          <t>125464</t>
+        </is>
+      </c>
+      <c r="D395" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Side Light (Blue) - 125464</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F395" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 11525845; listing says oven/range light component, models not shown - verify</t>
         </is>
       </c>
     </row>
     <row r="396">
-      <c r="A396" s="4" t="inlineStr">
+      <c r="A396" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B396" s="4" t="n">
+      <c r="B396" s="3" t="n">
         <v>9656525</v>
       </c>
-      <c r="C396" s="4" t="inlineStr"/>
-      <c r="D396" s="4" t="inlineStr"/>
-      <c r="E396" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F396" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C396" s="3" t="inlineStr"/>
+      <c r="D396" s="3" t="inlineStr"/>
+      <c r="E396" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F396" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="397">
-      <c r="A397" s="4" t="inlineStr">
+      <c r="A397" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B397" s="4" t="n">
+      <c r="B397" s="3" t="n">
         <v>9656545</v>
       </c>
-      <c r="C397" s="4" t="inlineStr"/>
-      <c r="D397" s="4" t="inlineStr"/>
-      <c r="E397" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F397" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C397" s="3" t="inlineStr"/>
+      <c r="D397" s="3" t="inlineStr"/>
+      <c r="E397" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F397" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="398">
-      <c r="A398" s="4" t="inlineStr">
+      <c r="A398" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B398" s="4" t="n">
+      <c r="B398" s="3" t="n">
         <v>9656558</v>
       </c>
-      <c r="C398" s="4" t="inlineStr"/>
-      <c r="D398" s="4" t="inlineStr"/>
-      <c r="E398" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F398" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C398" s="3" t="inlineStr">
+        <is>
+          <t>125166</t>
+        </is>
+      </c>
+      <c r="D398" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Oven Door (Burgundy Red) - 125166</t>
+        </is>
+      </c>
+      <c r="E398" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F398" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 9656558; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
     </row>
     <row r="399">
-      <c r="A399" s="4" t="inlineStr">
+      <c r="A399" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B399" s="4" t="n">
+      <c r="B399" s="3" t="n">
         <v>9656608</v>
       </c>
-      <c r="C399" s="4" t="inlineStr"/>
-      <c r="D399" s="4" t="inlineStr"/>
-      <c r="E399" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F399" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C399" s="3" t="inlineStr"/>
+      <c r="D399" s="3" t="inlineStr"/>
+      <c r="E399" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F399" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="400">
-      <c r="A400" s="4" t="inlineStr">
+      <c r="A400" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B400" s="4" t="n">
+      <c r="B400" s="3" t="n">
         <v>9656624</v>
       </c>
-      <c r="C400" s="4" t="inlineStr"/>
-      <c r="D400" s="4" t="inlineStr"/>
-      <c r="E400" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F400" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C400" s="3" t="inlineStr"/>
+      <c r="D400" s="3" t="inlineStr"/>
+      <c r="E400" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F400" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="401">
-      <c r="A401" s="4" t="inlineStr">
+      <c r="A401" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B401" s="4" t="n">
+      <c r="B401" s="3" t="n">
         <v>9656526</v>
       </c>
-      <c r="C401" s="4" t="inlineStr"/>
-      <c r="D401" s="4" t="inlineStr"/>
-      <c r="E401" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F401" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C401" s="3" t="inlineStr"/>
+      <c r="D401" s="3" t="inlineStr"/>
+      <c r="E401" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F401" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="402">
-      <c r="A402" s="4" t="inlineStr">
+      <c r="A402" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B402" s="4" t="n">
+      <c r="B402" s="3" t="n">
         <v>9656634</v>
       </c>
-      <c r="C402" s="4" t="inlineStr"/>
-      <c r="D402" s="4" t="inlineStr"/>
-      <c r="E402" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F402" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C402" s="3" t="inlineStr"/>
+      <c r="D402" s="3" t="inlineStr"/>
+      <c r="E402" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F402" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="403">
-      <c r="A403" s="4" t="inlineStr">
+      <c r="A403" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B403" s="4" t="n">
+      <c r="B403" s="3" t="n">
         <v>9656611</v>
       </c>
-      <c r="C403" s="4" t="inlineStr"/>
-      <c r="D403" s="4" t="inlineStr"/>
-      <c r="E403" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F403" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C403" s="3" t="inlineStr"/>
+      <c r="D403" s="3" t="inlineStr"/>
+      <c r="E403" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F403" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="404">
-      <c r="A404" s="4" t="inlineStr">
+      <c r="A404" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B404" s="4" t="n">
+      <c r="B404" s="3" t="n">
         <v>9656626</v>
       </c>
-      <c r="C404" s="4" t="inlineStr"/>
-      <c r="D404" s="4" t="inlineStr"/>
-      <c r="E404" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F404" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C404" s="3" t="inlineStr">
+        <is>
+          <t>125337</t>
+        </is>
+      </c>
+      <c r="D404" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Oven Door (Orange) - 125337</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F404" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 9656626; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
     </row>
     <row r="405">
-      <c r="A405" s="4" t="inlineStr">
+      <c r="A405" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B405" s="4" t="n">
+      <c r="B405" s="3" t="n">
         <v>9656562</v>
       </c>
-      <c r="C405" s="4" t="inlineStr"/>
-      <c r="D405" s="4" t="inlineStr"/>
-      <c r="E405" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F405" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C405" s="3" t="inlineStr"/>
+      <c r="D405" s="3" t="inlineStr"/>
+      <c r="E405" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F405" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="406">
-      <c r="A406" s="4" t="inlineStr">
+      <c r="A406" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B406" s="4" t="n">
+      <c r="B406" s="2" t="n">
         <v>9656680</v>
       </c>
-      <c r="C406" s="4" t="inlineStr"/>
-      <c r="D406" s="4" t="inlineStr"/>
-      <c r="E406" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F406" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C406" s="2" t="inlineStr">
+        <is>
+          <t>200477</t>
+        </is>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Work Table - 200477</t>
+        </is>
+      </c>
+      <c r="E406" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="inlineStr">
+        <is>
+          <t>Encompass item 9656680; fits PRO486/MAS486 range models per listing</t>
         </is>
       </c>
     </row>
     <row r="407">
-      <c r="A407" s="4" t="inlineStr">
+      <c r="A407" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B407" s="4" t="n">
+      <c r="B407" s="3" t="n">
         <v>9656598</v>
       </c>
-      <c r="C407" s="4" t="inlineStr"/>
-      <c r="D407" s="4" t="inlineStr"/>
-      <c r="E407" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F407" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C407" s="3" t="inlineStr"/>
+      <c r="D407" s="3" t="inlineStr"/>
+      <c r="E407" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F407" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="408">
-      <c r="A408" s="4" t="inlineStr">
+      <c r="A408" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B408" s="4" t="n">
+      <c r="B408" s="3" t="n">
         <v>9656610</v>
       </c>
-      <c r="C408" s="4" t="inlineStr"/>
-      <c r="D408" s="4" t="inlineStr"/>
-      <c r="E408" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F408" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C408" s="3" t="inlineStr"/>
+      <c r="D408" s="3" t="inlineStr"/>
+      <c r="E408" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F408" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="409">
-      <c r="A409" s="4" t="inlineStr">
+      <c r="A409" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B409" s="4" t="n">
+      <c r="B409" s="3" t="n">
         <v>9656630</v>
       </c>
-      <c r="C409" s="4" t="inlineStr"/>
-      <c r="D409" s="4" t="inlineStr"/>
-      <c r="E409" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F409" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C409" s="3" t="inlineStr"/>
+      <c r="D409" s="3" t="inlineStr"/>
+      <c r="E409" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F409" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="410">
-      <c r="A410" s="4" t="inlineStr">
+      <c r="A410" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B410" s="4" t="n">
+      <c r="B410" s="3" t="n">
         <v>9656635</v>
       </c>
-      <c r="C410" s="4" t="inlineStr"/>
-      <c r="D410" s="4" t="inlineStr"/>
-      <c r="E410" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F410" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C410" s="3" t="inlineStr"/>
+      <c r="D410" s="3" t="inlineStr"/>
+      <c r="E410" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F410" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="411">
-      <c r="A411" s="4" t="inlineStr">
+      <c r="A411" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B411" s="4" t="n">
+      <c r="B411" s="3" t="n">
         <v>9656697</v>
       </c>
-      <c r="C411" s="4" t="inlineStr"/>
-      <c r="D411" s="4" t="inlineStr"/>
-      <c r="E411" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F411" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C411" s="3" t="inlineStr"/>
+      <c r="D411" s="3" t="inlineStr"/>
+      <c r="E411" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F411" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="412">
-      <c r="A412" s="4" t="inlineStr">
+      <c r="A412" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B412" s="4" t="n">
+      <c r="B412" s="3" t="n">
         <v>9656554</v>
       </c>
-      <c r="C412" s="4" t="inlineStr"/>
-      <c r="D412" s="4" t="inlineStr"/>
-      <c r="E412" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F412" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C412" s="3" t="inlineStr"/>
+      <c r="D412" s="3" t="inlineStr"/>
+      <c r="E412" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F412" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="413">
-      <c r="A413" s="4" t="inlineStr">
+      <c r="A413" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B413" s="4" t="n">
+      <c r="B413" s="3" t="n">
         <v>9656564</v>
       </c>
-      <c r="C413" s="4" t="inlineStr"/>
-      <c r="D413" s="4" t="inlineStr"/>
-      <c r="E413" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F413" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C413" s="3" t="inlineStr"/>
+      <c r="D413" s="3" t="inlineStr"/>
+      <c r="E413" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F413" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="414">
-      <c r="A414" s="4" t="inlineStr">
+      <c r="A414" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B414" s="4" t="n">
+      <c r="B414" s="3" t="n">
         <v>9656600</v>
       </c>
-      <c r="C414" s="4" t="inlineStr"/>
-      <c r="D414" s="4" t="inlineStr"/>
-      <c r="E414" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F414" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C414" s="3" t="inlineStr">
+        <is>
+          <t>125311</t>
+        </is>
+      </c>
+      <c r="D414" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Oven Door Left (Burgundy Red) - 125311</t>
+        </is>
+      </c>
+      <c r="E414" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F414" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 9656600; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
     </row>
     <row r="415">
-      <c r="A415" s="4" t="inlineStr">
+      <c r="A415" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B415" s="4" t="n">
+      <c r="B415" s="3" t="n">
         <v>9656606</v>
       </c>
-      <c r="C415" s="4" t="inlineStr"/>
-      <c r="D415" s="4" t="inlineStr"/>
-      <c r="E415" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F415" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C415" s="3" t="inlineStr"/>
+      <c r="D415" s="3" t="inlineStr"/>
+      <c r="E415" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F415" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="416">
-      <c r="A416" s="4" t="inlineStr">
+      <c r="A416" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B416" s="4" t="n">
+      <c r="B416" s="3" t="n">
         <v>9656612</v>
       </c>
-      <c r="C416" s="4" t="inlineStr"/>
-      <c r="D416" s="4" t="inlineStr"/>
-      <c r="E416" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F416" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C416" s="3" t="inlineStr"/>
+      <c r="D416" s="3" t="inlineStr"/>
+      <c r="E416" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F416" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="417">
-      <c r="A417" s="4" t="inlineStr">
+      <c r="A417" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B417" s="4" t="n">
+      <c r="B417" s="3" t="n">
         <v>9656596</v>
       </c>
-      <c r="C417" s="4" t="inlineStr"/>
-      <c r="D417" s="4" t="inlineStr"/>
-      <c r="E417" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F417" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C417" s="3" t="inlineStr"/>
+      <c r="D417" s="3" t="inlineStr"/>
+      <c r="E417" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F417" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="418">
-      <c r="A418" s="4" t="inlineStr">
+      <c r="A418" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B418" s="4" t="n">
+      <c r="B418" s="3" t="n">
         <v>9656607</v>
       </c>
-      <c r="C418" s="4" t="inlineStr"/>
-      <c r="D418" s="4" t="inlineStr"/>
-      <c r="E418" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F418" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C418" s="3" t="inlineStr"/>
+      <c r="D418" s="3" t="inlineStr"/>
+      <c r="E418" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F418" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="419">
-      <c r="A419" s="4" t="inlineStr">
+      <c r="A419" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B419" s="4" t="n">
+      <c r="B419" s="3" t="n">
         <v>9657402</v>
       </c>
-      <c r="C419" s="4" t="inlineStr"/>
-      <c r="D419" s="4" t="inlineStr"/>
-      <c r="E419" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F419" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C419" s="3" t="inlineStr"/>
+      <c r="D419" s="3" t="inlineStr"/>
+      <c r="E419" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F419" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="420">
-      <c r="A420" s="4" t="inlineStr">
+      <c r="A420" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B420" s="4" t="n">
+      <c r="B420" s="3" t="n">
         <v>9656623</v>
       </c>
-      <c r="C420" s="4" t="inlineStr"/>
-      <c r="D420" s="4" t="inlineStr"/>
-      <c r="E420" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F420" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C420" s="3" t="inlineStr">
+        <is>
+          <t>125334</t>
+        </is>
+      </c>
+      <c r="D420" s="3" t="inlineStr">
+        <is>
+          <t>Bertazzoni Range Oven Door (Orange) - 125334</t>
+        </is>
+      </c>
+      <c r="E420" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F420" s="3" t="inlineStr">
+        <is>
+          <t>Encompass item 9656623; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
     </row>
     <row r="421">
-      <c r="A421" s="4" t="inlineStr">
+      <c r="A421" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B421" s="4" t="n">
+      <c r="B421" s="3" t="n">
         <v>9656628</v>
       </c>
-      <c r="C421" s="4" t="inlineStr"/>
-      <c r="D421" s="4" t="inlineStr"/>
-      <c r="E421" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F421" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C421" s="3" t="inlineStr"/>
+      <c r="D421" s="3" t="inlineStr"/>
+      <c r="E421" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F421" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="422">
-      <c r="A422" s="4" t="inlineStr">
+      <c r="A422" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B422" s="4" t="n">
+      <c r="B422" s="3" t="n">
         <v>9657974</v>
       </c>
-      <c r="C422" s="4" t="inlineStr"/>
-      <c r="D422" s="4" t="inlineStr"/>
-      <c r="E422" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F422" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C422" s="3" t="inlineStr"/>
+      <c r="D422" s="3" t="inlineStr"/>
+      <c r="E422" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F422" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>
     <row r="423">
-      <c r="A423" s="4" t="inlineStr">
+      <c r="A423" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B423" s="4" t="n">
+      <c r="B423" s="3" t="n">
         <v>9657971</v>
       </c>
-      <c r="C423" s="4" t="inlineStr"/>
-      <c r="D423" s="4" t="inlineStr"/>
-      <c r="E423" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="F423" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: number is an Encompass item ID and needs lookup</t>
+      <c r="C423" s="3" t="inlineStr"/>
+      <c r="D423" s="3" t="inlineStr"/>
+      <c r="E423" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="F423" s="3" t="inlineStr">
+        <is>
+          <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Range collection: add Encompass item URLs for unresolved rows
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +27,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -59,11 +63,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F476"/>
+  <dimension ref="A1:G476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -438,6 +443,7 @@
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="90" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,6 +477,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Encompass item URL (to look up PN)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -553,6 +564,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11595960/</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -605,6 +621,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12642965/</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -627,6 +648,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11436689/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -739,6 +765,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12753806/</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -761,6 +792,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10611278/</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -783,6 +819,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10680596/</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -805,6 +846,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10680596/</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -827,6 +873,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12680098/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -849,6 +900,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/7890960/</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -871,6 +927,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679883/</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -893,6 +954,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10404403/</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -975,6 +1041,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11436677/</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -997,6 +1068,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10157279/</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1019,6 +1095,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10611794/</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1041,6 +1122,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10886963/</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1123,6 +1209,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11436042/</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1145,6 +1236,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11435736/</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1257,6 +1353,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11058274/</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1309,6 +1410,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11061297/</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1331,6 +1437,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11058222/</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1383,6 +1494,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10886968/</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1435,6 +1551,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10675475/</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -1457,6 +1578,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10674712/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1479,6 +1605,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10676272/</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -1501,6 +1632,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10674702/</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1523,6 +1659,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10675426/</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -1545,6 +1686,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10610180/</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1597,6 +1743,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10600408/</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1649,6 +1800,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10611357/</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -1671,6 +1827,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10310172/</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1723,6 +1884,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10309304/</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -1775,6 +1941,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10159065/</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -1797,6 +1968,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510323/</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -1819,6 +1995,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9435695/</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -1841,6 +2022,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10734397/</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -1863,6 +2049,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12585182/</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -1885,6 +2076,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510219/</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -1907,6 +2103,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510330/</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -1929,6 +2130,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510541/</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -1951,6 +2157,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510324/</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -1973,6 +2184,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510542/</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -1995,6 +2211,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13358549/</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -2017,6 +2238,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13358551/</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -2039,6 +2265,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13358536/</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -2061,6 +2292,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751712/</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -2083,6 +2319,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12611420/</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2135,6 +2376,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12313536/</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -2157,6 +2403,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12313556/</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -2179,6 +2430,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12421850/</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -2201,6 +2457,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679668/</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -2223,6 +2484,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12421793/</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -2245,6 +2511,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12542405/</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -2267,6 +2538,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12928938/</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -2289,6 +2565,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929193/</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -2311,6 +2592,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13073385/</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -2333,6 +2619,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679686/</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2385,6 +2676,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679871/</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2437,6 +2733,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12421798/</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -2459,6 +2760,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679702/</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -2481,6 +2787,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751631/</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -2503,6 +2814,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929115/</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
@@ -2525,6 +2841,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679898/</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -2547,6 +2868,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679691/</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
@@ -2569,6 +2895,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12542403/</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -2591,6 +2922,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929173/</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -2613,6 +2949,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679884/</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -2635,6 +2976,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13343026/</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
@@ -2657,6 +3003,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12421792/</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -2679,6 +3030,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679868/</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
@@ -2701,6 +3057,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12672966/</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -2723,6 +3084,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929168/</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
@@ -2745,6 +3111,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751677/</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -2767,6 +3138,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751630/</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -2789,6 +3165,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751688/</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -2811,6 +3192,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12642607/</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -2893,6 +3279,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12672967/</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -2915,6 +3306,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12672338/</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
@@ -2937,6 +3333,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12674283/</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -2959,6 +3360,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12674277/</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
@@ -2981,6 +3387,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11832725/</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -3003,6 +3414,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12298458/</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
@@ -3025,6 +3441,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11597472/</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -3047,6 +3468,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13072364/</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -3069,6 +3495,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510645/</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -3091,6 +3522,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12675415/</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
@@ -3113,6 +3549,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G112" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12329123/</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -3135,6 +3576,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11433914/</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
@@ -3157,6 +3603,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G114" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11435787/</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -3179,6 +3630,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10611282/</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -3261,6 +3717,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G118" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11432514/</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -3283,6 +3744,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11432299/</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
@@ -3305,6 +3771,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G120" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9442266/</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -3327,6 +3798,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929862/</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -3349,6 +3825,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12680089/</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -3371,6 +3852,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679903/</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
@@ -3393,6 +3879,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679900/</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -3445,6 +3936,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11073939/</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -3467,6 +3963,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10676447/</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
@@ -3489,6 +3990,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9320062/</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -3511,6 +4017,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11666804/</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -3593,6 +4104,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G132" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11074017/</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -3615,6 +4131,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G133" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510592/</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
@@ -3637,6 +4158,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12680125/</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -3689,6 +4215,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11074016/</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -3711,6 +4242,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G137" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679700/</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
@@ -3733,6 +4269,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12588659/</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -3755,6 +4296,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G139" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679867/</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
@@ -3777,6 +4323,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G140" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12674291/</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -3799,6 +4350,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G141" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12928911/</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
@@ -3821,6 +4377,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G142" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12624036/</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -3843,6 +4404,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G143" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13023562/</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
@@ -3865,6 +4431,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G144" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929665/</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -3887,6 +4458,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G145" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510445/</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
@@ -3909,6 +4485,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G146" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12627343/</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -3931,6 +4512,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G147" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679913/</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
@@ -3953,6 +4539,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G148" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13343028/</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -3975,6 +4566,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G149" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12307932/</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -4027,6 +4623,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G151" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929167/</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
@@ -4049,6 +4650,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G152" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751680/</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -4071,6 +4677,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G153" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751674/</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
@@ -4093,6 +4704,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G154" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12627353/</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
@@ -4115,6 +4731,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G155" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751558/</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
@@ -4137,6 +4758,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G156" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12627495/</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -4159,6 +4785,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G157" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12680086/</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
@@ -4181,6 +4812,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G158" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12421774/</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -4203,6 +4839,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G159" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12680048/</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
@@ -4225,6 +4866,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751559/</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -4247,6 +4893,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G161" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679689/</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
@@ -4269,6 +4920,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G162" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12680107/</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -4291,6 +4947,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G163" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9892353/</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
@@ -4313,6 +4974,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G164" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9892346/</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -4335,6 +5001,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G165" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9890274/</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -4387,6 +5058,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G167" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9884707/</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
@@ -4439,6 +5115,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G169" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9451966/</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
@@ -4551,6 +5232,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G173" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9442710/</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
@@ -4573,6 +5259,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G174" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9441456/</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -4595,6 +5286,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G175" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9441453/</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -4647,6 +5343,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G177" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9439424/</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
@@ -4669,6 +5370,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G178" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9439422/</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -4781,6 +5487,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G182" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9415736/</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -4803,6 +5514,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G183" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9314383/</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -4885,6 +5601,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G186" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9222258/</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -4967,6 +5688,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G189" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/8182806/</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -5079,6 +5805,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G193" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12971639/</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
@@ -5101,6 +5832,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G194" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12751690/</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -5123,6 +5859,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G195" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12675514/</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
@@ -5145,6 +5886,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G196" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12673051/</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
@@ -5167,6 +5913,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G197" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12585181/</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="3" t="inlineStr">
@@ -5189,6 +5940,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G198" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12322643/</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
@@ -5211,6 +5967,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G199" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12329076/</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
@@ -5233,6 +5994,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G200" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12299586/</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
@@ -5255,6 +6021,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G201" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12299399/</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="3" t="inlineStr">
@@ -5277,6 +6048,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G202" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11831685/</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -5359,6 +6135,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G205" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11500937/</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -5411,6 +6192,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G207" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11436685/</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="3" t="inlineStr">
@@ -5433,6 +6219,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G208" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11436676/</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
@@ -5485,6 +6276,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G210" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679722/</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
@@ -5507,6 +6303,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G211" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510440/</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="3" t="inlineStr">
@@ -5529,6 +6330,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G212" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11510439/</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
@@ -5551,6 +6357,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G213" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12733984/</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="3" t="inlineStr">
@@ -5573,6 +6384,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G214" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929116/</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
@@ -5595,6 +6411,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G215" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12925362/</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -5677,6 +6498,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G218" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9657361/</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
@@ -5699,6 +6525,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G219" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656609/</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="3" t="inlineStr">
@@ -5721,6 +6552,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G220" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656674/</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
@@ -5743,6 +6579,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G221" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656567/</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="3" t="inlineStr">
@@ -5765,6 +6606,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G222" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656550/</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
@@ -5787,6 +6633,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G223" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319081/</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="3" t="inlineStr">
@@ -5809,6 +6660,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G224" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319074/</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="3" t="inlineStr">
@@ -5831,6 +6687,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G225" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319073/</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="3" t="inlineStr">
@@ -5853,6 +6714,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G226" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319099/</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="3" t="inlineStr">
@@ -5875,6 +6741,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G227" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319087/</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="3" t="inlineStr">
@@ -5897,6 +6768,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G228" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319089/</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
@@ -5919,6 +6795,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G229" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584933/</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="3" t="inlineStr">
@@ -5941,6 +6822,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G230" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584913/</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="3" t="inlineStr">
@@ -5963,6 +6849,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G231" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584931/</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="3" t="inlineStr">
@@ -6015,6 +6906,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G233" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10681415/</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="3" t="inlineStr">
@@ -6037,6 +6933,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G234" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10178316/</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="3" t="inlineStr">
@@ -6089,6 +6990,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G236" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12320902/</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
@@ -6111,6 +7017,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G237" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12320894/</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="3" t="inlineStr">
@@ -6133,6 +7044,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G238" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12925667/</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="3" t="inlineStr">
@@ -6155,6 +7071,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G239" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12499168/</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="3" t="inlineStr">
@@ -6177,6 +7098,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G240" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12488483/</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
@@ -6199,6 +7125,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G241" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12709500/</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="3" t="inlineStr">
@@ -6247,6 +7178,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G243" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11053978/</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="3" t="inlineStr">
@@ -6269,6 +7205,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G244" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598732/</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="3" t="inlineStr">
@@ -6291,6 +7232,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G245" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12282197/</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="3" t="inlineStr">
@@ -6313,6 +7259,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G246" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598731/</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
@@ -6335,6 +7286,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G247" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12444669/</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -6387,6 +7343,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G249" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11597884/</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="3" t="inlineStr">
@@ -6409,6 +7370,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G250" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12469969/</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="3" t="inlineStr">
@@ -6431,6 +7397,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G251" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6953935/</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="3" t="inlineStr">
@@ -6453,6 +7424,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G252" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11580852/</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="3" t="inlineStr">
@@ -6475,6 +7451,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G253" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11577484/</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="3" t="inlineStr">
@@ -6497,6 +7478,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G254" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10074064/</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="3" t="inlineStr">
@@ -6519,6 +7505,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G255" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10130655/</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="3" t="inlineStr">
@@ -6541,6 +7532,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G256" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10168871/</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="3" t="inlineStr">
@@ -6563,6 +7559,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G257" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10168894/</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -6615,6 +7616,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G259" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10838321/</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="3" t="inlineStr">
@@ -6637,6 +7643,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G260" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10847437/</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="3" t="inlineStr">
@@ -6659,6 +7670,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G261" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10868484/</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="3" t="inlineStr">
@@ -6681,6 +7697,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G262" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10878840/</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="3" t="inlineStr">
@@ -6733,6 +7754,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G264" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11053935/</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="inlineStr">
@@ -6755,6 +7781,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G265" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11114498/</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="3" t="inlineStr">
@@ -6807,6 +7838,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G267" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11535419/</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="3" t="inlineStr">
@@ -6829,6 +7865,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G268" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11578315/</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="3" t="inlineStr">
@@ -6851,6 +7892,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G269" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11593512/</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -6903,6 +7949,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G271" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598251/</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="3" t="inlineStr">
@@ -6925,6 +7976,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G272" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598730/</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="3" t="inlineStr">
@@ -6947,6 +8003,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G273" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598733/</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="3" t="inlineStr">
@@ -6969,6 +8030,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G274" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598735/</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="3" t="inlineStr">
@@ -6991,6 +8057,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G275" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598514/</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="3" t="inlineStr">
@@ -7013,6 +8084,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G276" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11654521/</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="3" t="inlineStr">
@@ -7035,6 +8111,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G277" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11742617/</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -7117,6 +8198,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G280" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12501545/</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="3" t="inlineStr">
@@ -7139,6 +8225,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G281" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12499976/</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="3" t="inlineStr">
@@ -7161,6 +8252,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G282" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12619548/</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -7213,6 +8309,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G284" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12924181/</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="3" t="inlineStr">
@@ -7235,6 +8336,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G285" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12924176/</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
@@ -7287,6 +8393,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G287" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6862572/</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -7339,6 +8450,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G289" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6947174/</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="3" t="inlineStr">
@@ -7361,6 +8477,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G290" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6953830/</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="3" t="inlineStr">
@@ -7383,6 +8504,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G291" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6947945/</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="3" t="inlineStr">
@@ -7405,6 +8531,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G292" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6948923/</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="3" t="inlineStr">
@@ -7427,6 +8558,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G293" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/8089749/</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -7479,6 +8615,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G295" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9328045/</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="3" t="inlineStr">
@@ -7501,6 +8642,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G296" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9331494/</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -7553,6 +8699,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G298" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9350706/</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="3" t="inlineStr">
@@ -7575,6 +8726,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G299" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349281/</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="3" t="inlineStr">
@@ -7597,6 +8753,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G300" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349682/</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="3" t="inlineStr">
@@ -7619,6 +8780,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G301" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835037/</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="3" t="inlineStr">
@@ -7641,6 +8807,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G302" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835005/</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="3" t="inlineStr">
@@ -7663,6 +8834,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G303" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835061/</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="3" t="inlineStr">
@@ -7685,6 +8861,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G304" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349282/</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="3" t="inlineStr">
@@ -7707,6 +8888,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G305" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349296/</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="3" t="inlineStr">
@@ -7729,6 +8915,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G306" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349191/</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -7811,6 +9002,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G309" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349290/</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -7863,6 +9059,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G311" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835004/</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="3" t="inlineStr">
@@ -7885,6 +9086,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G312" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835036/</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="3" t="inlineStr">
@@ -7907,6 +9113,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G313" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835062/</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="3" t="inlineStr">
@@ -7929,6 +9140,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G314" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349047/</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="3" t="inlineStr">
@@ -7951,6 +9167,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G315" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11654923/</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="3" t="inlineStr">
@@ -7973,6 +9194,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G316" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11578959/</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="3" t="inlineStr">
@@ -7995,6 +9221,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G317" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11579003/</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="3" t="inlineStr">
@@ -8017,6 +9248,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G318" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10848443/</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="3" t="inlineStr">
@@ -8039,6 +9275,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G319" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12432120/</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="3" t="inlineStr">
@@ -8061,6 +9302,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G320" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12537681/</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="3" t="inlineStr">
@@ -8083,6 +9329,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G321" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12616076/</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="3" t="inlineStr">
@@ -8105,6 +9356,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G322" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12616092/</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="3" t="inlineStr">
@@ -8157,6 +9413,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G324" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12574883/</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="3" t="inlineStr">
@@ -8179,6 +9440,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G325" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12444096/</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="3" t="inlineStr">
@@ -8201,6 +9467,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G326" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11830416/</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
@@ -8253,6 +9524,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G328" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12524352/</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -8305,6 +9581,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G330" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12444423/</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="3" t="inlineStr">
@@ -8327,6 +9608,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G331" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11579255/</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
@@ -8379,6 +9665,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G333" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12598403/</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
@@ -8461,6 +9752,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G336" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12924782/</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="3" t="inlineStr">
@@ -8483,6 +9779,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G337" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12492721/</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
@@ -8535,6 +9836,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G339" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12934311/</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="3" t="inlineStr">
@@ -8557,6 +9863,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G340" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12585179/</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
@@ -8609,6 +9920,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G342" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/7018146/</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="3" t="inlineStr">
@@ -8631,6 +9947,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G343" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11437542/</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="3" t="inlineStr">
@@ -8653,6 +9974,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G344" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13372326/</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="3" t="inlineStr">
@@ -8675,6 +10001,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G345" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12923012/</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="3" t="inlineStr">
@@ -8697,6 +10028,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G346" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12923009/</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="3" t="inlineStr">
@@ -8719,6 +10055,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G347" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13070534/</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="3" t="inlineStr">
@@ -8741,6 +10082,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G348" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/14899112/</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="3" t="inlineStr">
@@ -8763,6 +10109,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G349" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13609473/</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="3" t="inlineStr">
@@ -8785,6 +10136,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G350" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12323195/</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="3" t="inlineStr">
@@ -8807,6 +10163,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G351" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12488482/</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="3" t="inlineStr">
@@ -8829,6 +10190,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G352" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12490537/</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="3" t="inlineStr">
@@ -8851,6 +10217,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G353" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12491052/</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="3" t="inlineStr">
@@ -8873,6 +10244,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G354" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12493839/</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="3" t="inlineStr">
@@ -8895,6 +10271,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G355" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12493851/</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="3" t="inlineStr">
@@ -8917,6 +10298,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G356" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12494273/</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="3" t="inlineStr">
@@ -8939,6 +10325,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G357" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12497106/</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="3" t="inlineStr">
@@ -8961,6 +10352,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G358" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12502886/</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
@@ -9013,6 +10409,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G360" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12503044/</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="3" t="inlineStr">
@@ -9035,6 +10436,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G361" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11525725/</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="3" t="inlineStr">
@@ -9057,6 +10463,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G362" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11598061/</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="3" t="inlineStr">
@@ -9079,6 +10490,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G363" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/14894572/</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="3" t="inlineStr">
@@ -9101,6 +10517,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G364" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/14894506/</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="3" t="inlineStr">
@@ -9123,6 +10544,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G365" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/14894576/</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="3" t="inlineStr">
@@ -9145,6 +10571,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G366" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/14896732/</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="3" t="inlineStr">
@@ -9167,6 +10598,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G367" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13589307/</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="3" t="inlineStr">
@@ -9189,6 +10625,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G368" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12709492/</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="3" t="inlineStr">
@@ -9211,6 +10652,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G369" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12709498/</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="3" t="inlineStr">
@@ -9233,6 +10679,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G370" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12709509/</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="3" t="inlineStr">
@@ -9255,6 +10706,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G371" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13393136/</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="3" t="inlineStr">
@@ -9277,6 +10733,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G372" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12934247/</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="3" t="inlineStr">
@@ -9299,6 +10760,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G373" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12934269/</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="3" t="inlineStr">
@@ -9321,6 +10787,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G374" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584900/</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="3" t="inlineStr">
@@ -9343,6 +10814,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G375" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584917/</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="3" t="inlineStr">
@@ -9365,6 +10841,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G376" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584929/</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="3" t="inlineStr">
@@ -9387,6 +10868,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G377" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584915/</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="3" t="inlineStr">
@@ -9409,6 +10895,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G378" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584920/</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="3" t="inlineStr">
@@ -9431,6 +10922,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G379" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584897/</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
@@ -9483,6 +10979,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G381" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584928/</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="3" t="inlineStr">
@@ -9505,6 +11006,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G382" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12320940/</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="3" t="inlineStr">
@@ -9527,6 +11033,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G383" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12320899/</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="3" t="inlineStr">
@@ -9549,6 +11060,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G384" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584904/</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="3" t="inlineStr">
@@ -9571,6 +11087,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G385" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584919/</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
@@ -9623,6 +11144,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G387" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319103/</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="3" t="inlineStr">
@@ -9645,6 +11171,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G388" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319088/</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="3" t="inlineStr">
@@ -9697,6 +11228,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G390" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12320897/</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="3" t="inlineStr">
@@ -9719,6 +11255,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G391" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319095/</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="3" t="inlineStr">
@@ -9741,6 +11282,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G392" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319101/</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="3" t="inlineStr">
@@ -9763,6 +11309,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G393" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12607236/</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="3" t="inlineStr">
@@ -9785,6 +11336,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G394" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12524602/</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="3" t="inlineStr">
@@ -9837,6 +11393,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G396" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656525/</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="3" t="inlineStr">
@@ -9859,6 +11420,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G397" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656545/</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="3" t="inlineStr">
@@ -9911,6 +11477,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G399" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656608/</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="3" t="inlineStr">
@@ -9933,6 +11504,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G400" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656624/</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="3" t="inlineStr">
@@ -9955,6 +11531,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G401" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656526/</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="3" t="inlineStr">
@@ -9977,6 +11558,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G402" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656634/</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="3" t="inlineStr">
@@ -9999,6 +11585,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G403" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656611/</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="3" t="inlineStr">
@@ -10051,6 +11642,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G405" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656562/</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
@@ -10103,6 +11699,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G407" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656598/</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="3" t="inlineStr">
@@ -10125,6 +11726,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G408" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656610/</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="3" t="inlineStr">
@@ -10147,6 +11753,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G409" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656630/</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" s="3" t="inlineStr">
@@ -10169,6 +11780,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G410" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656635/</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" s="3" t="inlineStr">
@@ -10191,6 +11807,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G411" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656697/</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" s="3" t="inlineStr">
@@ -10213,6 +11834,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G412" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656554/</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="3" t="inlineStr">
@@ -10235,6 +11861,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G413" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656564/</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="3" t="inlineStr">
@@ -10287,6 +11918,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G415" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656606/</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" s="3" t="inlineStr">
@@ -10309,6 +11945,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G416" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656612/</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" s="3" t="inlineStr">
@@ -10331,6 +11972,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G417" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656596/</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" s="3" t="inlineStr">
@@ -10353,6 +11999,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G418" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656607/</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" s="3" t="inlineStr">
@@ -10375,6 +12026,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G419" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9657402/</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" s="3" t="inlineStr">
@@ -10427,6 +12083,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G421" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656628/</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" s="3" t="inlineStr">
@@ -10449,6 +12110,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G422" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9657974/</t>
+        </is>
+      </c>
     </row>
     <row r="423">
       <c r="A423" s="3" t="inlineStr">
@@ -10471,6 +12137,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G423" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9657971/</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
@@ -10523,6 +12194,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G425" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6947174/</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" s="3" t="inlineStr">
@@ -10545,6 +12221,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G426" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349047/</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
@@ -10597,6 +12278,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G428" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6947945/</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" s="3" t="inlineStr">
@@ -10619,6 +12305,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G429" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/8089749/</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" s="3" t="inlineStr">
@@ -10641,6 +12332,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G430" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349296/</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" s="3" t="inlineStr">
@@ -10663,6 +12359,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G431" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11654521/</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" s="3" t="inlineStr">
@@ -10685,6 +12386,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G432" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349191/</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="3" t="inlineStr">
@@ -10707,6 +12413,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G433" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349282/</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" s="3" t="inlineStr">
@@ -10729,6 +12440,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G434" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349290/</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" s="3" t="inlineStr">
@@ -10751,6 +12467,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G435" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349682/</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
@@ -10803,6 +12524,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G437" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835061/</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
@@ -10855,6 +12581,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G439" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835036/</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" s="3" t="inlineStr">
@@ -10877,6 +12608,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G440" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835062/</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="3" t="inlineStr">
@@ -10899,6 +12635,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G441" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835005/</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="3" t="inlineStr">
@@ -10921,6 +12662,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G442" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835004/</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="3" t="inlineStr">
@@ -10943,6 +12689,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G443" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9350706/</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" s="3" t="inlineStr">
@@ -10965,6 +12716,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G444" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6948923/</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="3" t="inlineStr">
@@ -10987,6 +12743,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G445" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6953830/</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" s="3" t="inlineStr">
@@ -11009,6 +12770,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G446" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6953935/</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="3" t="inlineStr">
@@ -11061,6 +12827,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G448" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10168871/</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" s="3" t="inlineStr">
@@ -11083,6 +12854,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G449" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10878840/</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" s="3" t="inlineStr">
@@ -11105,6 +12881,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G450" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11577484/</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="3" t="inlineStr">
@@ -11127,6 +12908,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G451" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11578315/</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
@@ -11179,6 +12965,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G453" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11578959/</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="3" t="inlineStr">
@@ -11201,6 +12992,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G454" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11579003/</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" s="3" t="inlineStr">
@@ -11223,6 +13019,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G455" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11654923/</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="3" t="inlineStr">
@@ -11245,6 +13046,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G456" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12444423/</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="3" t="inlineStr">
@@ -11267,6 +13073,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G457" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12619548/</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="3" t="inlineStr">
@@ -11319,6 +13130,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G459" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11580852/</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" s="3" t="inlineStr">
@@ -11341,6 +13157,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G460" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10868484/</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="3" t="inlineStr">
@@ -11363,6 +13184,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G461" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12896729/</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="3" t="inlineStr">
@@ -11385,6 +13211,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G462" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12431317/</t>
+        </is>
+      </c>
     </row>
     <row r="463">
       <c r="A463" s="3" t="inlineStr">
@@ -11407,6 +13238,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G463" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10847437/</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" s="3" t="inlineStr">
@@ -11429,6 +13265,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G464" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10847476/</t>
+        </is>
+      </c>
     </row>
     <row r="465">
       <c r="A465" s="3" t="inlineStr">
@@ -11451,6 +13292,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G465" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9835037/</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" s="3" t="inlineStr">
@@ -11473,6 +13319,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G466" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11579255/</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" s="3" t="inlineStr">
@@ -11495,6 +13346,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G467" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12444096/</t>
+        </is>
+      </c>
     </row>
     <row r="468">
       <c r="A468" s="3" t="inlineStr">
@@ -11517,6 +13373,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G468" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12524352/</t>
+        </is>
+      </c>
     </row>
     <row r="469">
       <c r="A469" s="3" t="inlineStr">
@@ -11539,6 +13400,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G469" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/13053983/</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" s="3" t="inlineStr">
@@ -11561,6 +13427,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G470" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10074064/</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" s="3" t="inlineStr">
@@ -11583,6 +13454,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G471" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10404972/</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" s="3" t="inlineStr">
@@ -11605,6 +13481,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G472" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11500979/</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" s="3" t="inlineStr">
@@ -11627,6 +13508,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G473" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11501153/</t>
+        </is>
+      </c>
     </row>
     <row r="474">
       <c r="A474" s="3" t="inlineStr">
@@ -11649,6 +13535,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G474" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11501085/</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" s="3" t="inlineStr">
@@ -11671,6 +13562,11 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G475" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11057620/</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" s="3" t="inlineStr">
@@ -11693,8 +13589,393 @@
           <t>Number is an Encompass item ID, not a manufacturer part number; no matching Encompass page found by web search</t>
         </is>
       </c>
+      <c r="G476" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11501343/</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G124" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G126" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G129" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G132" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G133" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G134" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G138" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G139" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G141" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G142" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G144" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G145" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G146" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G148" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G149" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G151" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G152" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G153" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G154" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G155" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G156" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G157" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G158" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G159" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G160" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G161" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G162" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G163" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G164" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G165" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G167" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G169" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G173" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G174" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G175" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G177" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G178" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G182" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G183" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G186" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G189" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G193" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G194" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G195" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G196" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G197" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G198" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G199" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G201" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G202" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G205" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G207" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G208" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G210" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G211" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G212" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G213" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G214" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G215" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G218" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G219" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G220" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G221" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G222" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G223" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G224" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G225" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G226" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G227" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G228" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G229" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G230" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G231" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G233" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G234" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G236" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G237" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G238" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G239" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G240" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G241" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G243" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G244" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G245" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G246" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G247" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G249" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G250" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G251" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G252" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G253" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G254" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G255" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G256" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G257" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G259" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G260" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G261" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G262" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G264" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G267" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G268" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G269" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G271" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G272" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G273" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G274" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G275" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G276" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G277" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G282" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G284" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G285" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G287" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G289" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G290" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G293" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G295" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G296" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G298" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G299" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G300" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G301" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G302" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G303" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G304" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G305" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G306" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G309" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G311" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G312" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G313" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G314" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G315" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G316" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G317" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G318" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G319" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G320" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G321" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G322" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G324" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G325" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G326" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G328" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G330" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G331" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G333" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G337" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G339" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G340" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G342" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G343" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G344" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G345" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G348" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G349" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G350" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G351" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G352" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G357" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G358" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G363" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G364" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G365" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G366" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G367" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G368" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G369" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G370" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G371" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G372" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G373" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G374" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G375" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G376" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G377" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G378" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G379" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G381" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G382" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G383" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G384" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G385" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G387" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G388" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G390" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G391" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G392" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G393" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G394" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G396" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G397" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G399" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G400" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G401" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G402" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G403" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G405" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G407" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G408" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G409" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G410" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G411" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G412" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G413" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G415" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G416" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G417" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G418" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G419" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G421" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G422" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G423" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G425" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G426" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G428" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G429" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G430" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G431" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G432" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G433" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G434" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G435" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G437" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G439" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G440" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G441" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G442" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G443" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G444" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G445" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G446" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G448" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G449" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G450" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G451" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G453" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G454" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G455" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G456" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G457" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G459" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G460" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G461" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G462" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G463" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G464" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G465" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G466" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G467" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G468" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G469" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G470" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G471" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G472" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G473" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G474" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G475" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G476" r:id="rId378"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Range collection: Encompass URL for every row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Range_Collection_H1_tags.xlsx
+++ b/Range_Collection_H1_tags.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Encompass item URL (to look up PN)</t>
+          <t>Encompass item URL</t>
         </is>
       </c>
     </row>
@@ -512,6 +512,11 @@
           <t>Encompass listing ID 9444117; Encompass name "Lcc190,pyro,gas" (gas range control)</t>
         </is>
       </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9444117/Whirlpool/WPW10424330/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -540,6 +545,11 @@
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 9442454; Encompass name "Ctrl-mrc-ele-cv-no"</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9442454/Whirlpool/WPW10340304/</t>
         </is>
       </c>
     </row>
@@ -599,6 +609,11 @@
           <t>Encompass listing ID 10887231; single source</t>
         </is>
       </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10887231/Whirlpool/W10877013/</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -683,6 +698,11 @@
           <t>Encompass listing ID 9432080</t>
         </is>
       </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9432080/Whirlpool/W10141009/</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -713,6 +733,11 @@
           <t>Encompass listing ID 11829363; description on two Encompass pages</t>
         </is>
       </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11829363/Whirlpool/W11175876/</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -741,6 +766,11 @@
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 10156277; two Encompass pages</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10156277/GE/WB27X21393/</t>
         </is>
       </c>
     </row>
@@ -989,6 +1019,11 @@
           <t>Encompass listing ID 8133922; single Encompass page</t>
         </is>
       </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/8133922/Whirlpool/WP8507P232-60/</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1017,6 +1052,11 @@
       <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 9441452; single Encompass page</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9441452/Whirlpool/W10314417/</t>
         </is>
       </c>
     </row>
@@ -1157,6 +1197,11 @@
           <t>Encompass listing ID 11435391; single Encompass page</t>
         </is>
       </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11435391/Whirlpool/W11050551/</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1185,6 +1230,11 @@
       <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 9441394; single Encompass page</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9441394/Whirlpool/WPW10312660/</t>
         </is>
       </c>
     </row>
@@ -1271,6 +1321,11 @@
           <t>Encompass listing ID 11435125; single Encompass page</t>
         </is>
       </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11435125/Whirlpool/W11039099/</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1301,6 +1356,11 @@
           <t>Encompass item 10933892; description is generic (Parts Assembly); fits LRE3061 range models</t>
         </is>
       </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10933892/LG/AGM73551660/</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1329,6 +1389,11 @@
       <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Encompass listing ID 10891704; listing name only "Cooktop"</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10891704/Whirlpool/W10814036/</t>
         </is>
       </c>
     </row>
@@ -1388,6 +1453,11 @@
           <t>Encompass item 11058280; fits LDE4411ST/LRE4211ST ranges per listing</t>
         </is>
       </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11058280/LG/AGU74969003/</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -1472,6 +1542,11 @@
           <t>Encompass listing ID 10886716; two Encompass pages</t>
         </is>
       </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10886716/Whirlpool/W10884488/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1529,6 +1604,11 @@
           <t>Encompass listing ID 10886969; single Encompass page</t>
         </is>
       </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10886969/Whirlpool/W10904904/</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -1721,6 +1801,11 @@
           <t>Encompass listing ID 10610337 (SP10610337 cross-reference)</t>
         </is>
       </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10610337/Whirlpool/WPW10778305/</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -1778,6 +1863,11 @@
           <t>Encompass listing ID 10611938; two Encompass pages</t>
         </is>
       </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10611938/Whirlpool/W10772617/</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -1862,6 +1952,11 @@
           <t>Encompass item 10310174; listed under LG oven/range parts</t>
         </is>
       </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10310174/LG/EBR80595311/</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -1919,6 +2014,11 @@
           <t>Encompass item 10254170; listing does not state appliance type (DE92 prefix suggests oven/range) - verify</t>
         </is>
       </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10254170/Samsung/DE92-03671A/</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -2354,6 +2454,11 @@
           <t>Encompass item 12679982; fits NE58/NX58 range models per listing</t>
         </is>
       </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12679982/Samsung/DG94-03837A/</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -2654,6 +2759,11 @@
           <t>Encompass item 12710308; fits NE63T8 range models per listing</t>
         </is>
       </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12710308/Samsung/DG90-01208A/</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -2711,6 +2821,11 @@
           <t>Encompass item 12929094; fits NE63T8711QN range per listing</t>
         </is>
       </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12929094/Samsung/DG94-03552H/</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -3227,6 +3342,11 @@
           <t>Encompass listing ID 11574168; listing name only "Cooktop"</t>
         </is>
       </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11574168/Whirlpool/W11178790/</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3255,6 +3375,11 @@
       <c r="F101" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 12276720; two pages</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12276720/Whirlpool/W11219379/</t>
         </is>
       </c>
     </row>
@@ -3665,6 +3790,11 @@
           <t>Encompass item 11581931; fits LG ranges (LSE4617ST etc.) per listing</t>
         </is>
       </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11581931/LG/AGU75049011/</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -3693,6 +3823,11 @@
       <c r="F117" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 11434431; single page</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11434431/Whirlpool/W10919303/</t>
         </is>
       </c>
     </row>
@@ -3914,6 +4049,11 @@
           <t>Encompass item 12611405; fits NX60T8711SS range per listing</t>
         </is>
       </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12611405/Samsung/DG94-03551B/</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -4052,6 +4192,11 @@
           <t>Encompass item 11073559; listing fits Samsung microwave models, not a range</t>
         </is>
       </c>
+      <c r="G130" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11073559/Samsung/DG47-00048B/</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -4080,6 +4225,11 @@
       <c r="F131" s="2" t="inlineStr">
         <is>
           <t>Encompass item 11073366; fits NE58K9850 range models per listing</t>
+        </is>
+      </c>
+      <c r="G131" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11073366/Samsung/DE92-03966B/</t>
         </is>
       </c>
     </row>
@@ -4193,6 +4343,11 @@
           <t>Encompass item 12657718; fits NE63T8111SS range per listing</t>
         </is>
       </c>
+      <c r="G135" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12657718/Samsung/DG94-03578K/</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
@@ -4601,6 +4756,11 @@
           <t>Encompass item 12680021; fits NX60A6111SS range per listing</t>
         </is>
       </c>
+      <c r="G150" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12680021/Samsung/DG94-03952K/</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -5036,6 +5196,11 @@
           <t>Encompass listing ID 9889686; two pages</t>
         </is>
       </c>
+      <c r="G166" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9889686/Whirlpool/WPW10586736/</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -5093,6 +5258,11 @@
           <t>Encompass item 9630366; listing does not state appliance type - verify</t>
         </is>
       </c>
+      <c r="G168" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9630366/LG/EBR73821006/</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -5150,6 +5320,11 @@
           <t>Encompass listing ID 9443754; listing name only "Cooktop"</t>
         </is>
       </c>
+      <c r="G170" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9443754/Whirlpool/WPW10396829/</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -5180,6 +5355,11 @@
           <t>Encompass listing ID 9443235; single page</t>
         </is>
       </c>
+      <c r="G171" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9443235/Whirlpool/W10365134/</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -5208,6 +5388,11 @@
       <c r="F172" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 9442761; single page (LCC195 board)</t>
+        </is>
+      </c>
+      <c r="G172" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9442761/Whirlpool/WPW10349742/</t>
         </is>
       </c>
     </row>
@@ -5321,6 +5506,11 @@
           <t>Encompass listing ID 9440666; single page</t>
         </is>
       </c>
+      <c r="G176" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9440666/Whirlpool/WPW10293048/</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -5405,6 +5595,11 @@
           <t>Encompass listing ID 9415744; single page</t>
         </is>
       </c>
+      <c r="G179" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9415744/Whirlpool/WP8507P236-60/</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -5435,6 +5630,11 @@
           <t>Encompass listing ID 9415741; two pages</t>
         </is>
       </c>
+      <c r="G180" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9415741/Whirlpool/WP8507P231-60/</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -5463,6 +5663,11 @@
       <c r="F181" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 9415739; single page</t>
+        </is>
+      </c>
+      <c r="G181" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9415739/Whirlpool/WP8507P229-60/</t>
         </is>
       </c>
     </row>
@@ -5549,6 +5754,11 @@
           <t>Encompass listing ID 9394490; single page</t>
         </is>
       </c>
+      <c r="G184" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9394490/Whirlpool/WP5760M302-60/</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -5577,6 +5787,11 @@
       <c r="F185" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 9250850; single page (Maytag-branded)</t>
+        </is>
+      </c>
+      <c r="G185" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9250850/Whirlpool/5701M760-60/</t>
         </is>
       </c>
     </row>
@@ -5636,6 +5851,11 @@
           <t>Encompass item 8254902; appliance type unclear in search (possibly dishwasher) - verify</t>
         </is>
       </c>
+      <c r="G187" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/8254902/LG/EBR64624601/</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
@@ -5664,6 +5884,11 @@
       <c r="F188" s="3" t="inlineStr">
         <is>
           <t>Encompass item 8253060; listed under HVAC room air - not a range part, verify</t>
+        </is>
+      </c>
+      <c r="G188" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/8253060/LG/EBR68349111/</t>
         </is>
       </c>
     </row>
@@ -5723,6 +5948,11 @@
           <t>Encompass listing ID 7038738; Encompass and Amazon pages</t>
         </is>
       </c>
+      <c r="G190" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/7038738/Whirlpool/WP9763716/</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -5753,6 +5983,11 @@
           <t>Encompass listing ID 7018145; three pages</t>
         </is>
       </c>
+      <c r="G191" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/7018145/Whirlpool/WP6610456/</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -5781,6 +6016,11 @@
       <c r="F192" s="2" t="inlineStr">
         <is>
           <t>Encompass item 6846510; fits LG range/cooktop models per listing</t>
+        </is>
+      </c>
+      <c r="G192" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6846510/LG/5300W1R009A/</t>
         </is>
       </c>
     </row>
@@ -6083,6 +6323,11 @@
           <t>Encompass item 11667430; listing does not state appliance type - verify</t>
         </is>
       </c>
+      <c r="G203" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11667430/Samsung/DG81-02239C/</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -6111,6 +6356,11 @@
       <c r="F204" s="2" t="inlineStr">
         <is>
           <t>Encompass item 11581929; fits LG ranges (LSE4617ST etc.) per listing</t>
+        </is>
+      </c>
+      <c r="G204" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11581929/LG/AGU75049010/</t>
         </is>
       </c>
     </row>
@@ -6170,6 +6420,11 @@
           <t>Encompass listing ID 11436692; single page</t>
         </is>
       </c>
+      <c r="G206" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11436692/Whirlpool/W11122557/</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -6254,6 +6509,11 @@
           <t>Encompass listing ID 11436503; only a repair Q&amp;A page names it, type not confirmed</t>
         </is>
       </c>
+      <c r="G209" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11436503/Whirlpool/W11113848/</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="3" t="inlineStr">
@@ -6446,6 +6706,11 @@
           <t>Encompass listing ID 9657916; replaces 910734</t>
         </is>
       </c>
+      <c r="G216" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9657916/Bertazzoni/910831/</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -6474,6 +6739,11 @@
       <c r="F217" s="2" t="inlineStr">
         <is>
           <t>Encompass listing ID 9657362; single page</t>
+        </is>
+      </c>
+      <c r="G217" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9657362/Bertazzoni/409050/</t>
         </is>
       </c>
     </row>
@@ -6884,6 +7154,11 @@
           <t>Encompass item 11584932; description is Bertazzoni catalog wording, appliance type not stated - verify</t>
         </is>
       </c>
+      <c r="G232" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584932/Bertazzoni/200559/</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="3" t="inlineStr">
@@ -6968,6 +7243,11 @@
           <t>Encompass item 12710552; appliance type not stated - verify</t>
         </is>
       </c>
+      <c r="G235" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12710552/Bertazzoni/211256/</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="3" t="inlineStr">
@@ -7156,6 +7436,11 @@
           <t>Only a forum thread links it to an Encompass listing for a Beko/Blomberg gas range; manufacturer part number not found</t>
         </is>
       </c>
+      <c r="G242" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11829909/</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
@@ -7321,6 +7606,11 @@
           <t>Encompass item 12499480; fits HBE5452UC series (built-in oven) per listing</t>
         </is>
       </c>
+      <c r="G248" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12499480/Bosch/11033919/</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="3" t="inlineStr">
@@ -7594,6 +7884,11 @@
           <t>Encompass listing ID 10387982; single page</t>
         </is>
       </c>
+      <c r="G258" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10387982/Fisher &amp; Paykel/210782P/</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="inlineStr">
@@ -7732,6 +8027,11 @@
           <t>Listing shows 10879182 as base part for model 807038640; single seller page</t>
         </is>
       </c>
+      <c r="G263" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10879182/Electrolux/807038640/</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="3" t="inlineStr">
@@ -7816,6 +8116,11 @@
           <t>Encompass item 11525561; Encompass description truncated ("Ignition D") and appliance type not stated - verify</t>
         </is>
       </c>
+      <c r="G266" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11525561/Bosch/00618624/</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
@@ -7927,6 +8232,11 @@
           <t>Encompass item 11596813; fits HBL8461UC/HBN8451UC oven models per listing</t>
         </is>
       </c>
+      <c r="G270" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11596813/Bosch/11020741/</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="3" t="inlineStr">
@@ -8146,6 +8456,11 @@
           <t>Encompass listing ID 12427085; single page</t>
         </is>
       </c>
+      <c r="G278" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12427085/GE/WB27X33137/</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="3" t="inlineStr">
@@ -8174,6 +8489,11 @@
       <c r="F279" s="3" t="inlineStr">
         <is>
           <t>Encompass item 12499289; listing fits mixed PRG/PRD dishwasher and oven models - verify appliance type</t>
+        </is>
+      </c>
+      <c r="G279" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12499289/Bosch/11032521/</t>
         </is>
       </c>
     </row>
@@ -8287,6 +8607,11 @@
           <t>Encompass listing ID 12632407; single page</t>
         </is>
       </c>
+      <c r="G283" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12632407/GE/WB27X39826/</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="3" t="inlineStr">
@@ -8371,6 +8696,11 @@
           <t>Encompass item 12924300; fits HGI8056UC/HGI8046UC models per listing</t>
         </is>
       </c>
+      <c r="G286" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12924300/Bosch/12037243/</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="3" t="inlineStr">
@@ -8428,6 +8758,11 @@
           <t>Encompass listing ID 6874796; three Encompass pages</t>
         </is>
       </c>
+      <c r="G288" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/6874796/GE/WB57K5/</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="3" t="inlineStr">
@@ -8593,6 +8928,11 @@
           <t>Encompass listing ID 9329006; two Encompass pages</t>
         </is>
       </c>
+      <c r="G294" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9329006/GE/WB27T11076/</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="3" t="inlineStr">
@@ -8677,6 +9017,11 @@
           <t>Encompass listing ID 9328760; three Encompass pages</t>
         </is>
       </c>
+      <c r="G297" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9328760/GE/WB27K10245/</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="3" t="inlineStr">
@@ -8950,6 +9295,11 @@
           <t>Encompass item 9349093; fits EW30 range models per listing</t>
         </is>
       </c>
+      <c r="G307" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349093/Electrolux/316443916/</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
@@ -8978,6 +9328,11 @@
       <c r="F308" s="2" t="inlineStr">
         <is>
           <t>Encompass item 9350269 listed under brand Electrolux; fits EW30 range models per listing</t>
+        </is>
+      </c>
+      <c r="G308" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9350269/Electrolux/316576610/</t>
         </is>
       </c>
     </row>
@@ -9037,6 +9392,11 @@
           <t>Encompass item 9350077 listed under brand Electrolux; fits FGGF-series ranges per listing</t>
         </is>
       </c>
+      <c r="G310" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9350077/Electrolux/316560118/</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="3" t="inlineStr">
@@ -9391,6 +9751,11 @@
           <t>Encompass item 10848602; listing shows refrigerator (ZDP) models, not a range - appliance type omitted, verify</t>
         </is>
       </c>
+      <c r="G323" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10848602/GE/WB24X24087/</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="3" t="inlineStr">
@@ -9502,6 +9867,11 @@
           <t>Encompass item 11578327 listed under brand Electrolux</t>
         </is>
       </c>
+      <c r="G327" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11578327/Electrolux/5304511258/</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="3" t="inlineStr">
@@ -9559,6 +9929,11 @@
           <t>Encompass item 12732070; fits GCRI/FGIH induction range models per listing</t>
         </is>
       </c>
+      <c r="G329" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12732070/Electrolux/5304527384/</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="3" t="inlineStr">
@@ -9643,6 +10018,11 @@
           <t>Encompass item 11830415 (blomberg.encompass.com listing)</t>
         </is>
       </c>
+      <c r="G332" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11830415/Blomberg/4410300337/</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="3" t="inlineStr">
@@ -9700,6 +10080,11 @@
           <t>Encompass item 11830418 (blomberg.encompass.com listing)</t>
         </is>
       </c>
+      <c r="G334" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11830418/Blomberg/4410600053/</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="3" t="inlineStr">
@@ -9728,6 +10113,11 @@
       <c r="F335" s="3" t="inlineStr">
         <is>
           <t>Encompass item 12487471; fits VTN/VTI models - appliance type not stated, verify</t>
+        </is>
+      </c>
+      <c r="G335" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12487471/Bosch/00669416/</t>
         </is>
       </c>
     </row>
@@ -9814,6 +10204,11 @@
           <t>Encompass item 12503030; fits HBL-series oven models per listing</t>
         </is>
       </c>
+      <c r="G338" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12503030/Bosch/20000554/</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="3" t="inlineStr">
@@ -9898,6 +10293,11 @@
           <t>Encompass item 10933730; listing describes oven control board for LG ranges</t>
         </is>
       </c>
+      <c r="G341" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10933730/LG/EBR77562705/</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="3" t="inlineStr">
@@ -10387,6 +10787,11 @@
           <t>Encompass item 12503043; fits HEI8056U oven models per listing</t>
         </is>
       </c>
+      <c r="G359" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12503043/Bosch/20000598/</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="3" t="inlineStr">
@@ -10957,6 +11362,11 @@
           <t>Encompass item 11584921; oven door, fits PROF486 range models per listing</t>
         </is>
       </c>
+      <c r="G380" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11584921/Bertazzoni/128027/</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="3" t="inlineStr">
@@ -11122,6 +11532,11 @@
           <t>Encompass item 12319102; fits PROF486 range models per listing</t>
         </is>
       </c>
+      <c r="G386" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319102/Bertazzoni/128027-DA/</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="3" t="inlineStr">
@@ -11206,6 +11621,11 @@
           <t>Encompass item 12319100; fitment models not shown - appliance type assumed from oven door family, verify</t>
         </is>
       </c>
+      <c r="G389" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/12319100/Bertazzoni/128021-DA/</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="3" t="inlineStr">
@@ -11371,6 +11791,11 @@
           <t>Encompass item 11525845; listing says oven/range light component, models not shown - verify</t>
         </is>
       </c>
+      <c r="G395" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11525845/Bertazzoni/125464/</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="3" t="inlineStr">
@@ -11455,6 +11880,11 @@
           <t>Encompass item 9656558; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
+      <c r="G398" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656558/Bertazzoni/125166/</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="3" t="inlineStr">
@@ -11620,6 +12050,11 @@
           <t>Encompass item 9656626; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
+      <c r="G404" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656626/Bertazzoni/125337/</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="3" t="inlineStr">
@@ -11677,6 +12112,11 @@
           <t>Encompass item 9656680; fits PRO486/MAS486 range models per listing</t>
         </is>
       </c>
+      <c r="G406" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656680/Bertazzoni/200477/</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" s="3" t="inlineStr">
@@ -11896,6 +12336,11 @@
           <t>Encompass item 9656600; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
+      <c r="G414" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656600/Bertazzoni/125311/</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" s="3" t="inlineStr">
@@ -12061,6 +12506,11 @@
           <t>Encompass item 9656623; fitment models not shown - appliance type assumed from oven door, verify</t>
         </is>
       </c>
+      <c r="G420" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9656623/Bertazzoni/125334/</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="3" t="inlineStr">
@@ -12172,6 +12622,11 @@
           <t>Encompass listing ID 10387982; single page</t>
         </is>
       </c>
+      <c r="G424" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10387982/Fisher &amp; Paykel/210782P/</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" s="3" t="inlineStr">
@@ -12256,6 +12711,11 @@
           <t>Encompass item 9349093; fits EW30 range models per listing</t>
         </is>
       </c>
+      <c r="G427" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9349093/Electrolux/316443916/</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" s="3" t="inlineStr">
@@ -12502,6 +12962,11 @@
           <t>Encompass item 9350077 listed under brand Electrolux; fits FGGF-series ranges per listing</t>
         </is>
       </c>
+      <c r="G436" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9350077/Electrolux/316560118/</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" s="3" t="inlineStr">
@@ -12559,6 +13024,11 @@
           <t>Encompass item 9350269 listed under brand Electrolux; fits EW30 range models per listing</t>
         </is>
       </c>
+      <c r="G438" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/9350269/Electrolux/316576610/</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="3" t="inlineStr">
@@ -12805,6 +13275,11 @@
           <t>Encompass item 10168877; listing names ES540 (range control) but no appliance type stated - verify</t>
         </is>
       </c>
+      <c r="G447" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10168877/Electrolux/5304495520/</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" s="3" t="inlineStr">
@@ -12943,6 +13418,11 @@
           <t>Encompass item 11578327 listed under brand Electrolux</t>
         </is>
       </c>
+      <c r="G452" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/11578327/Electrolux/5304511258/</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" s="3" t="inlineStr">
@@ -13108,6 +13588,11 @@
           <t>Listing shows 10879182 as base part for model 807038640; single seller page</t>
         </is>
       </c>
+      <c r="G458" s="4" t="inlineStr">
+        <is>
+          <t>https://encompass.com/item/10879182/Electrolux/807038640/</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="3" t="inlineStr">
@@ -13597,384 +14082,481 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G124" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G126" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G129" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G132" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G133" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G134" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G138" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G139" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G141" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G142" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G144" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G145" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G146" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G148" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G149" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G151" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G152" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G153" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G154" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G155" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G156" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G157" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G158" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G159" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G160" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G161" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G162" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G163" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G164" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G165" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G167" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G169" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G173" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G174" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G175" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G177" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G178" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G182" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G183" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G186" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G189" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G193" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G194" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G195" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G196" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G197" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G198" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G199" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G201" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G202" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G205" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G207" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G208" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G210" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G211" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G212" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G213" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G214" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G215" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G218" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G219" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G220" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G221" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G222" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G223" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G224" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G225" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G226" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G227" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G228" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G229" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G230" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G231" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G233" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G234" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G236" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G237" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G238" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G239" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G240" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G241" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G243" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G244" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G245" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G246" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G247" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G249" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G250" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G251" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G252" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G253" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G254" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G255" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G256" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G257" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G259" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G260" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G261" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G262" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G264" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G267" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G268" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G269" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G271" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G272" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G273" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G274" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G275" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G276" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G277" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G282" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G284" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G285" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G287" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G289" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G290" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G293" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G295" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G296" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G298" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G299" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G300" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G301" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G302" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G303" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G304" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G305" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G306" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G309" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G311" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G312" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G313" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G314" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G315" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G316" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G317" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G318" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G319" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G320" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G321" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G322" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G324" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G325" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G326" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G328" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G330" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G331" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G333" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G337" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G339" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G340" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G342" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G343" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G344" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G345" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G348" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G349" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G350" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G351" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G352" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G357" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G358" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G363" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G364" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G365" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G366" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G367" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G368" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G369" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G370" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G371" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G372" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G373" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G374" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G375" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G376" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G377" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G378" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G379" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G381" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G382" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G383" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G384" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G385" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G387" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G388" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G390" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G391" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G392" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G393" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G394" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G396" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G397" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G399" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G400" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G401" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G402" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G403" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G405" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G407" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G408" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G409" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G410" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G411" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G412" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G413" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G415" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G416" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G417" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G418" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G419" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G421" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G422" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G423" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G425" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G426" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G428" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G429" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G430" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G431" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G432" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G433" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G434" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G435" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G437" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G439" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G440" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G441" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G442" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G443" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G444" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G445" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G446" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G448" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G449" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G450" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G451" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G453" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G454" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G455" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G456" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G457" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G459" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G460" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G461" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G462" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G463" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G464" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G465" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G466" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G467" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G468" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G469" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G470" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G471" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G472" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G473" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G474" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G475" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G476" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G304" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G305" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G306" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G307" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G308" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G309" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G310" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G311" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G312" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G313" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G314" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G315" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G316" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G317" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G318" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G319" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G320" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G321" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G322" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G323" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G324" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G325" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G326" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G327" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G328" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G329" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G330" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G331" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G332" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G333" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G334" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G335" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G337" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G338" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G339" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G340" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G341" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G342" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G343" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G372" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G373" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G374" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G375" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G376" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G377" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G378" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G379" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G380" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G381" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G382" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G383" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G384" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G385" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G386" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G387" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G388" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G389" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G390" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G391" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G392" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G393" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G394" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G395" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G396" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G397" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G398" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G399" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G400" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G401" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G402" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G403" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G404" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G405" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G406" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G407" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G408" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G409" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G410" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G411" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G412" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G413" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G414" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G415" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G416" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G417" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G418" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G419" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G420" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G421" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G422" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G423" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G424" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G425" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G426" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G427" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G428" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G429" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G430" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G431" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G432" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G433" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G434" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G435" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G436" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G437" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G438" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G439" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G440" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G441" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G442" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G443" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G444" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G445" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G446" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G447" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G448" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G449" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G450" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G451" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G452" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G453" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G454" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G455" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G456" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G457" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G458" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G459" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G460" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G461" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G462" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G463" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G464" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G465" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G466" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G467" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G468" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G469" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G470" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G471" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G472" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G473" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G474" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G475" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G476" r:id="rId475"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>